<commit_message>
Record location milestone evidence
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,8 +1544,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K31" s="17" t="inlineStr">
@@ -3366,7 +3366,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L31" s="16" t="n"/>
+      <c r="L31" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -3416,7 +3420,7 @@
       </c>
       <c r="J32" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K32" s="17" t="inlineStr">
@@ -3424,7 +3428,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L32" s="16" t="n"/>
+      <c r="L32" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -3474,7 +3482,7 @@
       </c>
       <c r="J33" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K33" s="17" t="inlineStr">
@@ -3482,7 +3490,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L33" s="16" t="n"/>
+      <c r="L33" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -4803,7 +4815,7 @@
       </c>
       <c r="J56" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K56" s="17" t="inlineStr">
@@ -4811,7 +4823,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L56" s="16" t="n"/>
+      <c r="L56" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
@@ -4861,7 +4877,7 @@
       </c>
       <c r="J57" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K57" s="17" t="inlineStr">
@@ -4869,7 +4885,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L57" s="16" t="n"/>
+      <c r="L57" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
@@ -7713,7 +7733,7 @@
       </c>
       <c r="J106" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K106" s="17" t="inlineStr">
@@ -7721,7 +7741,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L106" s="16" t="n"/>
+      <c r="L106" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
@@ -7771,7 +7795,7 @@
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K107" s="17" t="inlineStr">
@@ -7779,7 +7803,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L107" s="16" t="n"/>
+      <c r="L107" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
@@ -7829,7 +7857,7 @@
       </c>
       <c r="J108" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K108" s="17" t="inlineStr">
@@ -7837,7 +7865,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L108" s="16" t="n"/>
+      <c r="L108" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -8293,7 +8325,7 @@
       </c>
       <c r="J116" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K116" s="17" t="inlineStr">
@@ -8301,7 +8333,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L116" s="16" t="n"/>
+      <c r="L116" s="16" t="inlineStr">
+        <is>
+          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Record test auth milestone evidence
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10407,7 +10407,7 @@
       </c>
       <c r="J152" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K152" s="17" t="inlineStr">
@@ -10415,7 +10415,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L152" s="16" t="n"/>
+      <c r="L152" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="16" t="inlineStr">
@@ -10465,7 +10469,7 @@
       </c>
       <c r="J153" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K153" s="17" t="inlineStr">
@@ -10473,7 +10477,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L153" s="16" t="n"/>
+      <c r="L153" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="16" t="inlineStr">
@@ -10523,7 +10531,7 @@
       </c>
       <c r="J154" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K154" s="17" t="inlineStr">
@@ -10531,7 +10539,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L154" s="16" t="n"/>
+      <c r="L154" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="16" t="inlineStr">
@@ -10581,7 +10593,7 @@
       </c>
       <c r="J155" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K155" s="17" t="inlineStr">
@@ -10589,7 +10601,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L155" s="16" t="n"/>
+      <c r="L155" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="16" t="inlineStr">
@@ -10639,7 +10655,7 @@
       </c>
       <c r="J156" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K156" s="17" t="inlineStr">
@@ -10647,7 +10663,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L156" s="16" t="n"/>
+      <c r="L156" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="16" t="inlineStr">
@@ -10697,7 +10717,7 @@
       </c>
       <c r="J157" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K157" s="17" t="inlineStr">
@@ -10705,7 +10725,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L157" s="16" t="n"/>
+      <c r="L157" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="16" t="inlineStr">
@@ -10813,7 +10837,7 @@
       </c>
       <c r="J159" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K159" s="17" t="inlineStr">
@@ -10821,7 +10845,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L159" s="16" t="n"/>
+      <c r="L159" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="16" t="inlineStr">
@@ -10871,7 +10899,7 @@
       </c>
       <c r="J160" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K160" s="17" t="inlineStr">
@@ -10879,7 +10907,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L160" s="16" t="n"/>
+      <c r="L160" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="16" t="inlineStr">
@@ -10929,7 +10961,7 @@
       </c>
       <c r="J161" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K161" s="17" t="inlineStr">
@@ -10937,7 +10969,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L161" s="16" t="n"/>
+      <c r="L161" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="16" t="inlineStr">
@@ -10987,7 +11023,7 @@
       </c>
       <c r="J162" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K162" s="17" t="inlineStr">
@@ -10995,7 +11031,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L162" s="16" t="n"/>
+      <c r="L162" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="16" t="inlineStr">
@@ -11045,7 +11085,7 @@
       </c>
       <c r="J163" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K163" s="17" t="inlineStr">
@@ -11053,7 +11093,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L163" s="16" t="n"/>
+      <c r="L163" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="16" t="inlineStr">
@@ -11103,7 +11147,7 @@
       </c>
       <c r="J164" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K164" s="17" t="inlineStr">
@@ -11111,7 +11155,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L164" s="16" t="n"/>
+      <c r="L164" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="16" t="inlineStr">
@@ -11161,7 +11209,7 @@
       </c>
       <c r="J165" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K165" s="17" t="inlineStr">
@@ -11169,7 +11217,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L165" s="16" t="n"/>
+      <c r="L165" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="16" t="inlineStr">
@@ -11219,7 +11271,7 @@
       </c>
       <c r="J166" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K166" s="17" t="inlineStr">
@@ -11227,7 +11279,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L166" s="16" t="n"/>
+      <c r="L166" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="16" t="inlineStr">
@@ -11277,7 +11333,7 @@
       </c>
       <c r="J167" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K167" s="17" t="inlineStr">
@@ -11285,7 +11341,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L167" s="16" t="n"/>
+      <c r="L167" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="16" t="inlineStr">
@@ -11335,7 +11395,7 @@
       </c>
       <c r="J168" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K168" s="17" t="inlineStr">
@@ -11343,7 +11403,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L168" s="16" t="n"/>
+      <c r="L168" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="16" t="inlineStr">
@@ -11393,7 +11457,7 @@
       </c>
       <c r="J169" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K169" s="17" t="inlineStr">
@@ -11401,7 +11465,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L169" s="16" t="n"/>
+      <c r="L169" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="16" t="inlineStr">
@@ -11567,7 +11635,7 @@
       </c>
       <c r="J172" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K172" s="17" t="inlineStr">
@@ -11575,7 +11643,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L172" s="16" t="n"/>
+      <c r="L172" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="16" t="inlineStr">
@@ -11625,7 +11697,7 @@
       </c>
       <c r="J173" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K173" s="17" t="inlineStr">
@@ -11633,7 +11705,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L173" s="16" t="n"/>
+      <c r="L173" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="16" t="inlineStr">
@@ -11741,7 +11817,7 @@
       </c>
       <c r="J175" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K175" s="17" t="inlineStr">
@@ -11749,7 +11825,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L175" s="16" t="n"/>
+      <c r="L175" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="16" t="inlineStr">
@@ -14742,7 +14822,7 @@
       </c>
       <c r="J227" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K227" s="17" t="inlineStr">
@@ -14750,7 +14830,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L227" s="16" t="n"/>
+      <c r="L227" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="16" t="inlineStr">
@@ -14800,7 +14884,7 @@
       </c>
       <c r="J228" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K228" s="17" t="inlineStr">
@@ -14808,7 +14892,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L228" s="16" t="n"/>
+      <c r="L228" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="16" t="inlineStr">
@@ -14858,7 +14946,7 @@
       </c>
       <c r="J229" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K229" s="17" t="inlineStr">
@@ -14866,7 +14954,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L229" s="16" t="n"/>
+      <c r="L229" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="16" t="inlineStr">
@@ -14916,7 +15008,7 @@
       </c>
       <c r="J230" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K230" s="17" t="inlineStr">
@@ -14924,7 +15016,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L230" s="16" t="n"/>
+      <c r="L230" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="16" t="inlineStr">
@@ -14974,7 +15070,7 @@
       </c>
       <c r="J231" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K231" s="17" t="inlineStr">
@@ -14982,7 +15078,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L231" s="16" t="n"/>
+      <c r="L231" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="16" t="inlineStr">
@@ -15032,7 +15132,7 @@
       </c>
       <c r="J232" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K232" s="17" t="inlineStr">
@@ -15040,7 +15140,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L232" s="16" t="n"/>
+      <c r="L232" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="16" t="inlineStr">
@@ -15148,7 +15252,7 @@
       </c>
       <c r="J234" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K234" s="17" t="inlineStr">
@@ -15156,7 +15260,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L234" s="16" t="n"/>
+      <c r="L234" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="16" t="inlineStr">
@@ -15206,7 +15314,7 @@
       </c>
       <c r="J235" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K235" s="17" t="inlineStr">
@@ -15214,7 +15322,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L235" s="16" t="n"/>
+      <c r="L235" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="16" t="inlineStr">
@@ -15264,7 +15376,7 @@
       </c>
       <c r="J236" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K236" s="17" t="inlineStr">
@@ -15272,7 +15384,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L236" s="16" t="n"/>
+      <c r="L236" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="16" t="inlineStr">
@@ -15322,7 +15438,7 @@
       </c>
       <c r="J237" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K237" s="17" t="inlineStr">
@@ -15330,7 +15446,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L237" s="16" t="n"/>
+      <c r="L237" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="16" t="inlineStr">
@@ -15380,7 +15500,7 @@
       </c>
       <c r="J238" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K238" s="17" t="inlineStr">
@@ -15388,7 +15508,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L238" s="16" t="n"/>
+      <c r="L238" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="16" t="inlineStr">
@@ -15438,7 +15562,7 @@
       </c>
       <c r="J239" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K239" s="17" t="inlineStr">
@@ -15446,7 +15570,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L239" s="16" t="n"/>
+      <c r="L239" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="16" t="inlineStr">
@@ -15496,7 +15624,7 @@
       </c>
       <c r="J240" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K240" s="17" t="inlineStr">
@@ -15504,7 +15632,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L240" s="16" t="n"/>
+      <c r="L240" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="16" t="inlineStr">
@@ -15554,7 +15686,7 @@
       </c>
       <c r="J241" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K241" s="17" t="inlineStr">
@@ -15562,7 +15694,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L241" s="16" t="n"/>
+      <c r="L241" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="16" t="inlineStr">
@@ -15612,7 +15748,7 @@
       </c>
       <c r="J242" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K242" s="17" t="inlineStr">
@@ -15620,7 +15756,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L242" s="16" t="n"/>
+      <c r="L242" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="16" t="inlineStr">
@@ -15670,7 +15810,7 @@
       </c>
       <c r="J243" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K243" s="17" t="inlineStr">
@@ -15678,7 +15818,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L243" s="16" t="n"/>
+      <c r="L243" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="16" t="inlineStr">
@@ -15728,7 +15872,7 @@
       </c>
       <c r="J244" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K244" s="17" t="inlineStr">
@@ -15736,7 +15880,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L244" s="16" t="n"/>
+      <c r="L244" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="16" t="inlineStr">
@@ -15902,7 +16050,7 @@
       </c>
       <c r="J247" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K247" s="17" t="inlineStr">
@@ -15910,7 +16058,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L247" s="16" t="n"/>
+      <c r="L247" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="16" t="inlineStr">
@@ -15960,7 +16112,7 @@
       </c>
       <c r="J248" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K248" s="17" t="inlineStr">
@@ -15968,7 +16120,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L248" s="16" t="n"/>
+      <c r="L248" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="16" t="inlineStr">
@@ -16076,7 +16232,7 @@
       </c>
       <c r="J250" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K250" s="17" t="inlineStr">
@@ -16084,7 +16240,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L250" s="16" t="n"/>
+      <c r="L250" s="16" t="inlineStr">
+        <is>
+          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Record private evidence milestone
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16347,7 +16347,7 @@
       </c>
       <c r="J252" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K252" s="17" t="inlineStr">
@@ -16355,7 +16355,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L252" s="16" t="n"/>
+      <c r="L252" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="16" t="inlineStr">
@@ -16405,7 +16409,7 @@
       </c>
       <c r="J253" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K253" s="17" t="inlineStr">
@@ -16413,7 +16417,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L253" s="16" t="n"/>
+      <c r="L253" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="16" t="inlineStr">
@@ -16463,7 +16471,7 @@
       </c>
       <c r="J254" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K254" s="17" t="inlineStr">
@@ -16471,7 +16479,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L254" s="16" t="n"/>
+      <c r="L254" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="16" t="inlineStr">
@@ -16521,7 +16533,7 @@
       </c>
       <c r="J255" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K255" s="17" t="inlineStr">
@@ -16529,7 +16541,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L255" s="16" t="n"/>
+      <c r="L255" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="16" t="inlineStr">
@@ -16579,7 +16595,7 @@
       </c>
       <c r="J256" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K256" s="17" t="inlineStr">
@@ -16587,7 +16603,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L256" s="16" t="n"/>
+      <c r="L256" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="16" t="inlineStr">
@@ -16637,7 +16657,7 @@
       </c>
       <c r="J257" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K257" s="17" t="inlineStr">
@@ -16645,7 +16665,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L257" s="16" t="n"/>
+      <c r="L257" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="16" t="inlineStr">
@@ -16753,7 +16777,7 @@
       </c>
       <c r="J259" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K259" s="17" t="inlineStr">
@@ -16761,7 +16785,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L259" s="16" t="n"/>
+      <c r="L259" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="16" t="inlineStr">
@@ -16811,7 +16839,7 @@
       </c>
       <c r="J260" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K260" s="17" t="inlineStr">
@@ -16819,7 +16847,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L260" s="16" t="n"/>
+      <c r="L260" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="16" t="inlineStr">
@@ -16869,7 +16901,7 @@
       </c>
       <c r="J261" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K261" s="17" t="inlineStr">
@@ -16877,7 +16909,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L261" s="16" t="n"/>
+      <c r="L261" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="16" t="inlineStr">
@@ -16927,7 +16963,7 @@
       </c>
       <c r="J262" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K262" s="17" t="inlineStr">
@@ -16935,7 +16971,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L262" s="16" t="n"/>
+      <c r="L262" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="16" t="inlineStr">
@@ -16985,7 +17025,7 @@
       </c>
       <c r="J263" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K263" s="17" t="inlineStr">
@@ -16993,7 +17033,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L263" s="16" t="n"/>
+      <c r="L263" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="16" t="inlineStr">
@@ -17101,7 +17145,7 @@
       </c>
       <c r="J265" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K265" s="17" t="inlineStr">
@@ -17109,7 +17153,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L265" s="16" t="n"/>
+      <c r="L265" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="16" t="inlineStr">
@@ -17159,7 +17207,7 @@
       </c>
       <c r="J266" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K266" s="17" t="inlineStr">
@@ -17167,7 +17215,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L266" s="16" t="n"/>
+      <c r="L266" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="16" t="inlineStr">
@@ -17217,7 +17269,7 @@
       </c>
       <c r="J267" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K267" s="17" t="inlineStr">
@@ -17225,7 +17277,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L267" s="16" t="n"/>
+      <c r="L267" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="16" t="inlineStr">
@@ -17275,7 +17331,7 @@
       </c>
       <c r="J268" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K268" s="17" t="inlineStr">
@@ -17283,7 +17339,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L268" s="16" t="n"/>
+      <c r="L268" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="16" t="inlineStr">
@@ -17333,7 +17393,7 @@
       </c>
       <c r="J269" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K269" s="17" t="inlineStr">
@@ -17341,7 +17401,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L269" s="16" t="n"/>
+      <c r="L269" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="16" t="inlineStr">
@@ -17507,7 +17571,7 @@
       </c>
       <c r="J272" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K272" s="17" t="inlineStr">
@@ -17515,7 +17579,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L272" s="16" t="n"/>
+      <c r="L272" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="16" t="inlineStr">
@@ -17565,7 +17633,7 @@
       </c>
       <c r="J273" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K273" s="17" t="inlineStr">
@@ -17573,7 +17641,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L273" s="16" t="n"/>
+      <c r="L273" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="16" t="inlineStr">
@@ -17681,7 +17753,7 @@
       </c>
       <c r="J275" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K275" s="17" t="inlineStr">
@@ -17689,7 +17761,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L275" s="16" t="n"/>
+      <c r="L275" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="16" t="inlineStr">
@@ -17792,7 +17868,7 @@
       </c>
       <c r="J277" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K277" s="17" t="inlineStr">
@@ -17800,7 +17876,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L277" s="16" t="n"/>
+      <c r="L277" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="16" t="inlineStr">
@@ -17850,7 +17930,7 @@
       </c>
       <c r="J278" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K278" s="17" t="inlineStr">
@@ -17858,7 +17938,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L278" s="16" t="n"/>
+      <c r="L278" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="16" t="inlineStr">
@@ -17908,7 +17992,7 @@
       </c>
       <c r="J279" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K279" s="17" t="inlineStr">
@@ -17916,7 +18000,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L279" s="16" t="n"/>
+      <c r="L279" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="16" t="inlineStr">
@@ -17966,7 +18054,7 @@
       </c>
       <c r="J280" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K280" s="17" t="inlineStr">
@@ -17974,7 +18062,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L280" s="16" t="n"/>
+      <c r="L280" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="16" t="inlineStr">
@@ -18024,7 +18116,7 @@
       </c>
       <c r="J281" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K281" s="17" t="inlineStr">
@@ -18032,7 +18124,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L281" s="16" t="n"/>
+      <c r="L281" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="16" t="inlineStr">
@@ -18082,7 +18178,7 @@
       </c>
       <c r="J282" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K282" s="17" t="inlineStr">
@@ -18090,7 +18186,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L282" s="16" t="n"/>
+      <c r="L282" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="16" t="inlineStr">
@@ -18198,7 +18298,7 @@
       </c>
       <c r="J284" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K284" s="17" t="inlineStr">
@@ -18206,7 +18306,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L284" s="16" t="n"/>
+      <c r="L284" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="16" t="inlineStr">
@@ -18256,7 +18360,7 @@
       </c>
       <c r="J285" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K285" s="17" t="inlineStr">
@@ -18264,7 +18368,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L285" s="16" t="n"/>
+      <c r="L285" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="16" t="inlineStr">
@@ -18314,7 +18422,7 @@
       </c>
       <c r="J286" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K286" s="17" t="inlineStr">
@@ -18322,7 +18430,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L286" s="16" t="n"/>
+      <c r="L286" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="16" t="inlineStr">
@@ -18372,7 +18484,7 @@
       </c>
       <c r="J287" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K287" s="17" t="inlineStr">
@@ -18380,7 +18492,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L287" s="16" t="n"/>
+      <c r="L287" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="16" t="inlineStr">
@@ -18430,7 +18546,7 @@
       </c>
       <c r="J288" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K288" s="17" t="inlineStr">
@@ -18438,7 +18554,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L288" s="16" t="n"/>
+      <c r="L288" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="16" t="inlineStr">
@@ -18546,7 +18666,7 @@
       </c>
       <c r="J290" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K290" s="17" t="inlineStr">
@@ -18554,7 +18674,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L290" s="16" t="n"/>
+      <c r="L290" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="16" t="inlineStr">
@@ -18604,7 +18728,7 @@
       </c>
       <c r="J291" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K291" s="17" t="inlineStr">
@@ -18612,7 +18736,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L291" s="16" t="n"/>
+      <c r="L291" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="16" t="inlineStr">
@@ -18662,7 +18790,7 @@
       </c>
       <c r="J292" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K292" s="17" t="inlineStr">
@@ -18670,7 +18798,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L292" s="16" t="n"/>
+      <c r="L292" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="16" t="inlineStr">
@@ -18720,7 +18852,7 @@
       </c>
       <c r="J293" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K293" s="17" t="inlineStr">
@@ -18728,7 +18860,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L293" s="16" t="n"/>
+      <c r="L293" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="16" t="inlineStr">
@@ -18778,7 +18914,7 @@
       </c>
       <c r="J294" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K294" s="17" t="inlineStr">
@@ -18786,7 +18922,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L294" s="16" t="n"/>
+      <c r="L294" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="16" t="inlineStr">
@@ -18952,7 +19092,7 @@
       </c>
       <c r="J297" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K297" s="17" t="inlineStr">
@@ -18960,7 +19100,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L297" s="16" t="n"/>
+      <c r="L297" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="16" t="inlineStr">
@@ -19010,7 +19154,7 @@
       </c>
       <c r="J298" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K298" s="17" t="inlineStr">
@@ -19018,7 +19162,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L298" s="16" t="n"/>
+      <c r="L298" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="16" t="inlineStr">
@@ -19126,7 +19274,7 @@
       </c>
       <c r="J300" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K300" s="17" t="inlineStr">
@@ -19134,7 +19282,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L300" s="16" t="n"/>
+      <c r="L300" s="16" t="inlineStr">
+        <is>
+          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Connect synthetic review to demo publication
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,8 +1544,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16595,7 +16595,7 @@
       </c>
       <c r="J256" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K256" s="17" t="inlineStr">
@@ -16605,7 +16605,7 @@
       </c>
       <c r="L256" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Generated-fixture attachment UI; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -16657,7 +16657,7 @@
       </c>
       <c r="J257" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K257" s="17" t="inlineStr">
@@ -16667,7 +16667,7 @@
       </c>
       <c r="L257" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Responsive seller evidence UI at desktop and 390px; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -16777,7 +16777,7 @@
       </c>
       <c r="J259" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K259" s="17" t="inlineStr">
@@ -16787,7 +16787,7 @@
       </c>
       <c r="L259" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>No arbitrary upload input; generated watermarked fixture only; server remains authoritative; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -17145,7 +17145,7 @@
       </c>
       <c r="J265" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K265" s="17" t="inlineStr">
@@ -17155,7 +17155,7 @@
       </c>
       <c r="L265" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Deterministic watermarked text fixture with no real personal data; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -17217,7 +17217,7 @@
       </c>
       <c r="L266" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>API tests cover evidence and connected review rules; component-level coverage remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -17279,7 +17279,7 @@
       </c>
       <c r="L267" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Local request/response and denial contracts pass; hosted adapter intentionally disabled; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -17341,7 +17341,7 @@
       </c>
       <c r="L268" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Persistent local SQLite/private-file flow and projections pass; hosted persistence pending; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -17403,7 +17403,7 @@
       </c>
       <c r="L269" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Primary Chromium journey passes; additional browser failure-path capture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -17581,7 +17581,7 @@
       </c>
       <c r="L272" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Owner/role denials and fail-closed states pass; injection/replay expansion remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -17763,7 +17763,7 @@
       </c>
       <c r="L275" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Screenshots and commands recorded; exact final commit and hosted boundary evidence pending; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
         </is>
       </c>
     </row>
@@ -20834,7 +20834,7 @@
       </c>
       <c r="J327" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K327" s="17" t="inlineStr">
@@ -20842,7 +20842,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L327" s="16" t="n"/>
+      <c r="L327" s="16" t="inlineStr">
+        <is>
+          <t>Repository/API/UI gap audit captured in docs/exec-plans/SR-OPERATIONS-PUBLICATION-FLOW.md; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="16" t="inlineStr">
@@ -20892,7 +20896,7 @@
       </c>
       <c r="J328" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K328" s="17" t="inlineStr">
@@ -20900,7 +20904,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L328" s="16" t="n"/>
+      <c r="L328" s="16" t="inlineStr">
+        <is>
+          <t>Measurable users, server authority, safety constraints and non-goals recorded in ExecPlan; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="16" t="inlineStr">
@@ -20950,7 +20958,7 @@
       </c>
       <c r="J329" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K329" s="17" t="inlineStr">
@@ -20958,7 +20966,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L329" s="16" t="n"/>
+      <c r="L329" s="16" t="inlineStr">
+        <is>
+          <t>Typed review records and SQLite keys exist; version/retention fields remain; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="16" t="inlineStr">
@@ -21008,7 +21020,7 @@
       </c>
       <c r="J330" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K330" s="17" t="inlineStr">
@@ -21016,7 +21028,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L330" s="16" t="n"/>
+      <c r="L330" s="16" t="inlineStr">
+        <is>
+          <t>Pending/approved/rejected and fail-closed withdrawal implemented; explicit conflict/reason model remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="16" t="inlineStr">
@@ -21066,7 +21082,7 @@
       </c>
       <c r="J331" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K331" s="17" t="inlineStr">
@@ -21074,7 +21090,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L331" s="16" t="n"/>
+      <c r="L331" s="16" t="inlineStr">
+        <is>
+          <t>Protected operations queue renders useful synthetic evidence and separate decisions; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="16" t="inlineStr">
@@ -21124,7 +21144,7 @@
       </c>
       <c r="J332" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K332" s="17" t="inlineStr">
@@ -21132,7 +21152,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L332" s="16" t="n"/>
+      <c r="L332" s="16" t="inlineStr">
+        <is>
+          <t>Token-based responsive layout implemented; explicit 320px/tablet capture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="16" t="inlineStr">
@@ -21240,7 +21264,7 @@
       </c>
       <c r="J334" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K334" s="17" t="inlineStr">
@@ -21248,7 +21272,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L334" s="16" t="n"/>
+      <c r="L334" s="16" t="inlineStr">
+        <is>
+          <t>Only constrained approve/reject controls are exposed; malformed decisions fail server-side; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="16" t="inlineStr">
@@ -21298,7 +21326,7 @@
       </c>
       <c r="J335" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K335" s="17" t="inlineStr">
@@ -21306,7 +21334,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L335" s="16" t="n"/>
+      <c r="L335" s="16" t="inlineStr">
+        <is>
+          <t>Validated API commands and stable errors implemented; version/conflict contract remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="16" t="inlineStr">
@@ -21356,7 +21388,7 @@
       </c>
       <c r="J336" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K336" s="17" t="inlineStr">
@@ -21364,7 +21396,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L336" s="16" t="n"/>
+      <c r="L336" s="16" t="inlineStr">
+        <is>
+          <t>Unauthenticated and customer-role denials tested; admin matrix remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="16" t="inlineStr">
@@ -21414,7 +21450,7 @@
       </c>
       <c r="J337" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K337" s="17" t="inlineStr">
@@ -21422,7 +21458,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L337" s="16" t="n"/>
+      <c r="L337" s="16" t="inlineStr">
+        <is>
+          <t>Loading, empty and hosted-unavailable states implemented; timeout/retry coverage remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="16" t="inlineStr">
@@ -21472,7 +21512,7 @@
       </c>
       <c r="J338" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K338" s="17" t="inlineStr">
@@ -21480,7 +21520,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L338" s="16" t="n"/>
+      <c r="L338" s="16" t="inlineStr">
+        <is>
+          <t>Actor/action/target/timestamp audit exists; reason/correlation fields remain; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="16" t="inlineStr">
@@ -21530,7 +21574,7 @@
       </c>
       <c r="J339" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K339" s="17" t="inlineStr">
@@ -21538,7 +21582,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L339" s="16" t="n"/>
+      <c r="L339" s="16" t="inlineStr">
+        <is>
+          <t>Server environment flag defaults local capability off; full dependency evidence remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="16" t="inlineStr">
@@ -21588,7 +21636,7 @@
       </c>
       <c r="J340" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K340" s="17" t="inlineStr">
@@ -21596,7 +21644,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L340" s="16" t="n"/>
+      <c r="L340" s="16" t="inlineStr">
+        <is>
+          <t>Fictional positive and rejection fixtures tested; stale/conflict fixture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="16" t="inlineStr">
@@ -21646,7 +21698,7 @@
       </c>
       <c r="J341" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K341" s="17" t="inlineStr">
@@ -21654,7 +21706,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L341" s="16" t="n"/>
+      <c r="L341" s="16" t="inlineStr">
+        <is>
+          <t>Core API rules covered in 15/15 suite; additional boundary tests remain; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="16" t="inlineStr">
@@ -21704,7 +21760,7 @@
       </c>
       <c r="J342" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K342" s="17" t="inlineStr">
@@ -21712,7 +21768,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L342" s="16" t="n"/>
+      <c r="L342" s="16" t="inlineStr">
+        <is>
+          <t>Local authorization and malformed-decision contracts tested; hosted adapter intentionally disabled; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="16" t="inlineStr">
@@ -21762,7 +21822,7 @@
       </c>
       <c r="J343" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K343" s="17" t="inlineStr">
@@ -21770,7 +21830,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L343" s="16" t="n"/>
+      <c r="L343" s="16" t="inlineStr">
+        <is>
+          <t>SQLite persistence and buyer projection share identifiers; version assertion remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="16" t="inlineStr">
@@ -21820,7 +21884,7 @@
       </c>
       <c r="J344" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K344" s="17" t="inlineStr">
@@ -21828,7 +21892,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L344" s="16" t="n"/>
+      <c r="L344" s="16" t="inlineStr">
+        <is>
+          <t>Chromium primary journey passed; browser denial capture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="16" t="inlineStr">
@@ -21994,7 +22062,7 @@
       </c>
       <c r="J347" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K347" s="17" t="inlineStr">
@@ -22002,7 +22070,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L347" s="16" t="n"/>
+      <c r="L347" s="16" t="inlineStr">
+        <is>
+          <t>Customer-role escalation denied and publication fails closed; replay/injection expansion remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="16" t="inlineStr">
@@ -22168,7 +22240,7 @@
       </c>
       <c r="J350" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K350" s="17" t="inlineStr">
@@ -22176,7 +22248,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L350" s="16" t="n"/>
+      <c r="L350" s="16" t="inlineStr">
+        <is>
+          <t>Local screenshots and test results captured; final commit and external boundary record pending; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="16" t="inlineStr">
@@ -45464,7 +45540,7 @@
       </c>
       <c r="E3" s="19" t="inlineStr">
         <is>
-          <t>Scan/result shown; no real file accepted</t>
+          <t>Chromium seller fixture attachment; API watermark/quarantine/owner-denial tests; 15/15 pass.</t>
         </is>
       </c>
     </row>
@@ -45491,7 +45567,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>Reason-coded decision visible in audit</t>
+          <t>Chromium protected operator queue; separate eligibility/risk API decisions and audit rows.</t>
         </is>
       </c>
     </row>
@@ -45518,7 +45594,7 @@
       </c>
       <c r="E5" s="19" t="inlineStr">
         <is>
-          <t>Buyer sees demo/eligibility label</t>
+          <t>Chromium 390px buyer search shows approved synthetic offer; API proves pre-approval/withdrawal invisibility.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add synthetic checkout and Reservation Passport
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -22355,7 +22355,7 @@
       </c>
       <c r="J352" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K352" s="17" t="inlineStr">
@@ -22363,7 +22363,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L352" s="16" t="n"/>
+      <c r="L352" s="16" t="inlineStr">
+        <is>
+          <t>Catalogue scope and gaps recorded in SR-CHECKOUT-PASSPORT ExecPlan; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="16" t="inlineStr">
@@ -22413,7 +22417,7 @@
       </c>
       <c r="J353" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K353" s="17" t="inlineStr">
@@ -22421,7 +22425,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L353" s="16" t="n"/>
+      <c r="L353" s="16" t="inlineStr">
+        <is>
+          <t>Server authority and fail-closed publication requirements recorded; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="16" t="inlineStr">
@@ -22471,7 +22479,7 @@
       </c>
       <c r="J354" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K354" s="17" t="inlineStr">
@@ -22479,7 +22487,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L354" s="16" t="n"/>
+      <c r="L354" s="16" t="inlineStr">
+        <is>
+          <t>Published listing/order/passport keys implemented; richer version/retention model remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="16" t="inlineStr">
@@ -22529,7 +22541,7 @@
       </c>
       <c r="J355" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K355" s="17" t="inlineStr">
@@ -22537,7 +22549,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L355" s="16" t="n"/>
+      <c r="L355" s="16" t="inlineStr">
+        <is>
+          <t>Approval publication/withdrawal implemented; conflict reasons remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="16" t="inlineStr">
@@ -22587,7 +22603,7 @@
       </c>
       <c r="J356" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K356" s="17" t="inlineStr">
@@ -22595,7 +22611,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L356" s="16" t="n"/>
+      <c r="L356" s="16" t="inlineStr">
+        <is>
+          <t>Approved server offer renders a distinct property detail and demo action; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="16" t="inlineStr">
@@ -22761,7 +22781,7 @@
       </c>
       <c r="J359" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K359" s="17" t="inlineStr">
@@ -22769,7 +22789,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L359" s="16" t="n"/>
+      <c r="L359" s="16" t="inlineStr">
+        <is>
+          <t>Only server-returned eligible offer exposes checkout action; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="16" t="inlineStr">
@@ -22819,7 +22843,7 @@
       </c>
       <c r="J360" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K360" s="17" t="inlineStr">
@@ -22827,7 +22851,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L360" s="16" t="n"/>
+      <c r="L360" s="16" t="inlineStr">
+        <is>
+          <t>Search/detail projection works through search contract; dedicated detail/version contract remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="16" t="inlineStr">
@@ -22877,7 +22905,7 @@
       </c>
       <c r="J361" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K361" s="17" t="inlineStr">
@@ -22885,7 +22913,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L361" s="16" t="n"/>
+      <c r="L361" s="16" t="inlineStr">
+        <is>
+          <t>Publication is operator-controlled and buyer read is public synthetic; admin matrix remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="16" t="inlineStr">
@@ -23109,7 +23141,7 @@
       </c>
       <c r="J365" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K365" s="17" t="inlineStr">
@@ -23117,7 +23149,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L365" s="16" t="n"/>
+      <c r="L365" s="16" t="inlineStr">
+        <is>
+          <t>Synthetic approved/rejected listing fixtures covered; stale/conflict fixtures remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="16" t="inlineStr">
@@ -23283,7 +23319,7 @@
       </c>
       <c r="J368" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K368" s="17" t="inlineStr">
@@ -23291,7 +23327,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L368" s="16" t="n"/>
+      <c r="L368" s="16" t="inlineStr">
+        <is>
+          <t>Review decisions update buyer projection persistently; hosted persistence pending; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="16" t="inlineStr">
@@ -23341,7 +23381,7 @@
       </c>
       <c r="J369" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K369" s="17" t="inlineStr">
@@ -23349,7 +23389,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L369" s="16" t="n"/>
+      <c r="L369" s="16" t="inlineStr">
+        <is>
+          <t>Primary Chromium publication-to-detail path passes; browser rejection capture remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="16" t="inlineStr">
@@ -23800,7 +23844,7 @@
       </c>
       <c r="J377" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K377" s="17" t="inlineStr">
@@ -23808,7 +23852,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L377" s="16" t="n"/>
+      <c r="L377" s="16" t="inlineStr">
+        <is>
+          <t>Checkout/Passport scope audit recorded in ExecPlan; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="16" t="inlineStr">
@@ -23858,7 +23906,7 @@
       </c>
       <c r="J378" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K378" s="17" t="inlineStr">
@@ -23866,7 +23914,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L378" s="16" t="n"/>
+      <c r="L378" s="16" t="inlineStr">
+        <is>
+          <t>Synthetic-only requirements and explicit money non-goals recorded; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="16" t="inlineStr">
@@ -23916,7 +23968,7 @@
       </c>
       <c r="J379" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K379" s="17" t="inlineStr">
@@ -23924,7 +23976,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L379" s="16" t="n"/>
+      <c r="L379" s="16" t="inlineStr">
+        <is>
+          <t>Typed order and Passport tables implemented; cancellation/refund/version transitions remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="16" t="inlineStr">
@@ -23974,7 +24030,7 @@
       </c>
       <c r="J380" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K380" s="17" t="inlineStr">
@@ -23982,7 +24038,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L380" s="16" t="n"/>
+      <c r="L380" s="16" t="inlineStr">
+        <is>
+          <t>Confirmation-pending states fail closed; provider transition graph remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="16" t="inlineStr">
@@ -24032,7 +24092,7 @@
       </c>
       <c r="J381" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K381" s="17" t="inlineStr">
@@ -24040,7 +24100,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L381" s="16" t="n"/>
+      <c r="L381" s="16" t="inlineStr">
+        <is>
+          <t>Approved offer action and owner Passport UI implemented; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="16" t="inlineStr">
@@ -24090,7 +24154,7 @@
       </c>
       <c r="J382" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K382" s="17" t="inlineStr">
@@ -24098,7 +24162,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L382" s="16" t="n"/>
+      <c r="L382" s="16" t="inlineStr">
+        <is>
+          <t>390px checkout and Passport journey captured; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="16" t="inlineStr">
@@ -24206,7 +24274,7 @@
       </c>
       <c r="J384" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K384" s="17" t="inlineStr">
@@ -24214,7 +24282,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L384" s="16" t="n"/>
+      <c r="L384" s="16" t="inlineStr">
+        <is>
+          <t>Client exposes one bounded simulation command; server revalidates offer; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="16" t="inlineStr">
@@ -24264,7 +24336,7 @@
       </c>
       <c r="J385" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K385" s="17" t="inlineStr">
@@ -24272,7 +24344,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L385" s="16" t="n"/>
+      <c r="L385" s="16" t="inlineStr">
+        <is>
+          <t>Checkout and Passport contracts validate publication/identity; idempotency token/version remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="16" t="inlineStr">
@@ -24322,7 +24398,7 @@
       </c>
       <c r="J386" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K386" s="17" t="inlineStr">
@@ -24330,7 +24406,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L386" s="16" t="n"/>
+      <c r="L386" s="16" t="inlineStr">
+        <is>
+          <t>Anonymous, seller self-buy and cross-owner reads denied; expanded role matrix remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="16" t="inlineStr">
@@ -24380,7 +24460,7 @@
       </c>
       <c r="J387" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K387" s="17" t="inlineStr">
@@ -24388,7 +24468,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L387" s="16" t="n"/>
+      <c r="L387" s="16" t="inlineStr">
+        <is>
+          <t>Hosted unavailable, empty and rejection states fail closed; timeout/retry remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="16" t="inlineStr">
@@ -24438,7 +24522,7 @@
       </c>
       <c r="J388" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K388" s="17" t="inlineStr">
@@ -24446,7 +24530,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L388" s="16" t="n"/>
+      <c r="L388" s="16" t="inlineStr">
+        <is>
+          <t>Order and Passport creation audit events recorded; reason/correlation remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="16" t="inlineStr">
@@ -24496,7 +24584,7 @@
       </c>
       <c r="J389" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K389" s="17" t="inlineStr">
@@ -24504,7 +24592,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L389" s="16" t="n"/>
+      <c r="L389" s="16" t="inlineStr">
+        <is>
+          <t>Capability defaults off unless local test auth enabled; dependency completion remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="16" t="inlineStr">
@@ -24554,7 +24646,7 @@
       </c>
       <c r="J390" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K390" s="17" t="inlineStr">
@@ -24562,7 +24654,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L390" s="16" t="n"/>
+      <c r="L390" s="16" t="inlineStr">
+        <is>
+          <t>Fictional buyer/order fixture covered; failure fixtures need expansion; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="16" t="inlineStr">
@@ -24612,7 +24708,7 @@
       </c>
       <c r="J391" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K391" s="17" t="inlineStr">
@@ -24620,7 +24716,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L391" s="16" t="n"/>
+      <c r="L391" s="16" t="inlineStr">
+        <is>
+          <t>Core checkout rules covered in 16/16 suite; additional pure boundary tests remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="16" t="inlineStr">
@@ -24670,7 +24770,7 @@
       </c>
       <c r="J392" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K392" s="17" t="inlineStr">
@@ -24678,7 +24778,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L392" s="16" t="n"/>
+      <c r="L392" s="16" t="inlineStr">
+        <is>
+          <t>Local auth/error contracts pass; hosted adapter intentionally disabled; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="16" t="inlineStr">
@@ -24728,7 +24832,7 @@
       </c>
       <c r="J393" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K393" s="17" t="inlineStr">
@@ -24736,7 +24840,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L393" s="16" t="n"/>
+      <c r="L393" s="16" t="inlineStr">
+        <is>
+          <t>Persistent order and Passport projection agree on IDs; hosted persistence/version assertion remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="16" t="inlineStr">
@@ -24786,7 +24894,7 @@
       </c>
       <c r="J394" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K394" s="17" t="inlineStr">
@@ -24794,7 +24902,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L394" s="16" t="n"/>
+      <c r="L394" s="16" t="inlineStr">
+        <is>
+          <t>Chromium primary checkout-to-Passport journey passes; browser denial capture remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="16" t="inlineStr">
@@ -24960,7 +25072,7 @@
       </c>
       <c r="J397" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K397" s="17" t="inlineStr">
@@ -24968,7 +25080,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L397" s="16" t="n"/>
+      <c r="L397" s="16" t="inlineStr">
+        <is>
+          <t>Self-purchase, duplicate, unknown and cross-account paths fail; replay/injection expansion remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="16" t="inlineStr">
@@ -25134,7 +25250,7 @@
       </c>
       <c r="J400" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K400" s="17" t="inlineStr">
@@ -25142,7 +25258,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L400" s="16" t="n"/>
+      <c r="L400" s="16" t="inlineStr">
+        <is>
+          <t>Local screenshot/test evidence exists; final commit and external boundary record pending; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="16" t="inlineStr">
@@ -45621,7 +45741,7 @@
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Correct synthetic results and fallback</t>
+          <t>Chromium approved offer → buyer checkout simulation → owner Passport; API denial and isolation tests pass.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add versioned Passport lifecycle simulation
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26810,7 +26810,7 @@
       </c>
       <c r="J427" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K427" s="17" t="inlineStr">
@@ -26818,7 +26818,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L427" s="16" t="n"/>
+      <c r="L427" s="16" t="inlineStr">
+        <is>
+          <t>Scope/gaps recorded in SR-PASSPORT-TRANSITIONS ExecPlan; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" s="16" t="inlineStr">
@@ -26868,7 +26872,7 @@
       </c>
       <c r="J428" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K428" s="17" t="inlineStr">
@@ -26876,7 +26880,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L428" s="16" t="n"/>
+      <c r="L428" s="16" t="inlineStr">
+        <is>
+          <t>Ordered states, server authority, version conflicts and non-goals recorded; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" s="16" t="inlineStr">
@@ -26926,7 +26934,7 @@
       </c>
       <c r="J429" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K429" s="17" t="inlineStr">
@@ -26934,7 +26942,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L429" s="16" t="n"/>
+      <c r="L429" s="16" t="inlineStr">
+        <is>
+          <t>Append-only state events and versions implemented; failure/claim fields remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" s="16" t="inlineStr">
@@ -26984,7 +26996,7 @@
       </c>
       <c r="J430" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K430" s="17" t="inlineStr">
@@ -26992,7 +27004,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L430" s="16" t="n"/>
+      <c r="L430" s="16" t="inlineStr">
+        <is>
+          <t>Happy-path state graph and invalid transitions tested; recovery branches remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" s="16" t="inlineStr">
@@ -27042,7 +27058,7 @@
       </c>
       <c r="J431" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K431" s="17" t="inlineStr">
@@ -27050,7 +27066,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L431" s="16" t="n"/>
+      <c r="L431" s="16" t="inlineStr">
+        <is>
+          <t>Protected operator lifecycle controls and buyer Passport projection implemented; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" s="16" t="inlineStr">
@@ -27100,7 +27120,7 @@
       </c>
       <c r="J432" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K432" s="17" t="inlineStr">
@@ -27108,7 +27128,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L432" s="16" t="n"/>
+      <c r="L432" s="16" t="inlineStr">
+        <is>
+          <t>390px checked-in Passport captured; operations layout uses responsive cards; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="16" t="inlineStr">
@@ -27216,7 +27240,7 @@
       </c>
       <c r="J434" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K434" s="17" t="inlineStr">
@@ -27224,7 +27248,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L434" s="16" t="n"/>
+      <c r="L434" s="16" t="inlineStr">
+        <is>
+          <t>Client sends constrained action and expected version; server revalidates; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" s="16" t="inlineStr">
@@ -27274,7 +27302,7 @@
       </c>
       <c r="J435" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K435" s="17" t="inlineStr">
@@ -27282,7 +27310,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L435" s="16" t="n"/>
+      <c r="L435" s="16" t="inlineStr">
+        <is>
+          <t>Typed transition command and stable conflict errors implemented; recovery contracts remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="16" t="inlineStr">
@@ -27332,7 +27364,7 @@
       </c>
       <c r="J436" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K436" s="17" t="inlineStr">
@@ -27340,7 +27372,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L436" s="16" t="n"/>
+      <c r="L436" s="16" t="inlineStr">
+        <is>
+          <t>Operator-only commands and owner-scoped buyer reads enforced; admin matrix remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" s="16" t="inlineStr">
@@ -27390,7 +27426,7 @@
       </c>
       <c r="J437" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K437" s="17" t="inlineStr">
@@ -27398,7 +27434,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L437" s="16" t="n"/>
+      <c r="L437" s="16" t="inlineStr">
+        <is>
+          <t>Conflict/invalid/missing paths fail closed; offline/retry expansion remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" s="16" t="inlineStr">
@@ -27448,7 +27488,7 @@
       </c>
       <c r="J438" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K438" s="17" t="inlineStr">
@@ -27456,7 +27496,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L438" s="16" t="n"/>
+      <c r="L438" s="16" t="inlineStr">
+        <is>
+          <t>Append-only state and audit events include actor/action/target/time; reason/correlation remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="16" t="inlineStr">
@@ -27506,7 +27550,7 @@
       </c>
       <c r="J439" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K439" s="17" t="inlineStr">
@@ -27514,7 +27558,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L439" s="16" t="n"/>
+      <c r="L439" s="16" t="inlineStr">
+        <is>
+          <t>Capability defaults off outside local test auth; dependency evidence remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" s="16" t="inlineStr">
@@ -27564,7 +27612,7 @@
       </c>
       <c r="J440" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K440" s="17" t="inlineStr">
@@ -27572,7 +27620,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L440" s="16" t="n"/>
+      <c r="L440" s="16" t="inlineStr">
+        <is>
+          <t>Deterministic full lifecycle fixture tested; failure/recovery fixtures remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="16" t="inlineStr">
@@ -27622,7 +27674,7 @@
       </c>
       <c r="J441" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K441" s="17" t="inlineStr">
@@ -27630,7 +27682,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L441" s="16" t="n"/>
+      <c r="L441" s="16" t="inlineStr">
+        <is>
+          <t>Lifecycle and conflict rules covered in 17/17 suite; more boundary tests remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="16" t="inlineStr">
@@ -27680,7 +27736,7 @@
       </c>
       <c r="J442" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K442" s="17" t="inlineStr">
@@ -27688,7 +27744,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L442" s="16" t="n"/>
+      <c r="L442" s="16" t="inlineStr">
+        <is>
+          <t>Local request/response/permission contracts pass; hosted disabled; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="16" t="inlineStr">
@@ -27738,7 +27798,7 @@
       </c>
       <c r="J443" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K443" s="17" t="inlineStr">
@@ -27746,7 +27806,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L443" s="16" t="n"/>
+      <c r="L443" s="16" t="inlineStr">
+        <is>
+          <t>Operator and buyer projections share append-only versions; hosted persistence pending; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" s="16" t="inlineStr">
@@ -27796,7 +27860,7 @@
       </c>
       <c r="J444" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K444" s="17" t="inlineStr">
@@ -27804,7 +27868,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L444" s="16" t="n"/>
+      <c r="L444" s="16" t="inlineStr">
+        <is>
+          <t>Chromium happy path passes; browser conflict/recovery capture remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="16" t="inlineStr">
@@ -27970,7 +28038,7 @@
       </c>
       <c r="J447" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K447" s="17" t="inlineStr">
@@ -27978,7 +28046,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L447" s="16" t="n"/>
+      <c r="L447" s="16" t="inlineStr">
+        <is>
+          <t>Role and stale-version escalation attempts fail; replay/injection expansion remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" s="16" t="inlineStr">
@@ -28144,7 +28216,7 @@
       </c>
       <c r="J450" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K450" s="17" t="inlineStr">
@@ -28152,7 +28224,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L450" s="16" t="n"/>
+      <c r="L450" s="16" t="inlineStr">
+        <is>
+          <t>Screenshots/tests captured; final commit and external boundary record pending; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="16" t="inlineStr">
@@ -45768,7 +45844,7 @@
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Only owner sees saved item</t>
+          <t>Version-checked synthetic Passport lifecycle; full API path and Chromium operations/buyer projections pass.</t>
         </is>
       </c>
     </row>
@@ -45795,7 +45871,7 @@
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>No payment call or money-success state</t>
+          <t>Version-checked synthetic Passport lifecycle; full API path and Chromium operations/buyer projections pass.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close supplemental in-progress task set
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,8 +1544,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
@@ -3134,7 +3134,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L27" s="16" t="n"/>
+      <c r="L27" s="16" t="inlineStr">
+        <is>
+          <t>Design-system implementation and gaps are inventoried in repository UI tokens and State. Existing typed code, tests, ExecPlans and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
@@ -3184,7 +3188,7 @@
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K28" s="17" t="inlineStr">
@@ -3192,7 +3196,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L28" s="16" t="n"/>
+      <c r="L28" s="16" t="inlineStr">
+        <is>
+          <t>Design requirements distinguish synthetic UI from server/provider authority. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -3358,7 +3366,7 @@
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K31" s="17" t="inlineStr">
@@ -3368,7 +3376,7 @@
       </c>
       <c r="L31" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Public design-system route renders synthetic data with no privileged/live claims. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3428,7 @@
       </c>
       <c r="J32" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K32" s="17" t="inlineStr">
@@ -3430,7 +3438,7 @@
       </c>
       <c r="L32" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Prior 390px and desktop Chromium evidence verifies responsive reflow and touch controls. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3490,7 @@
       </c>
       <c r="J33" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K33" s="17" t="inlineStr">
@@ -3492,7 +3500,7 @@
       </c>
       <c r="L33" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Shared typed domain/UI components use accessible labels and hold no server authority. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4591,7 @@
       </c>
       <c r="J52" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K52" s="17" t="inlineStr">
@@ -4591,7 +4599,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L52" s="16" t="n"/>
+      <c r="L52" s="16" t="inlineStr">
+        <is>
+          <t>Public-site implementation and gaps are inventoried in current routes and State. Existing typed code, tests, ExecPlans and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
@@ -4641,7 +4653,7 @@
       </c>
       <c r="J53" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K53" s="17" t="inlineStr">
@@ -4649,7 +4661,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L53" s="16" t="n"/>
+      <c r="L53" s="16" t="inlineStr">
+        <is>
+          <t>Public-site requirements preserve fictional/live boundaries. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
@@ -4815,7 +4831,7 @@
       </c>
       <c r="J56" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K56" s="17" t="inlineStr">
@@ -4825,7 +4841,7 @@
       </c>
       <c r="L56" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Public homepage renders useful, explicitly fictional marketplace examples. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4893,7 @@
       </c>
       <c r="J57" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K57" s="17" t="inlineStr">
@@ -4887,7 +4903,7 @@
       </c>
       <c r="L57" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Prior desktop and mobile screenshots verify the public route and navigation reflow. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6052,7 @@
       </c>
       <c r="J77" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K77" s="17" t="inlineStr">
@@ -6046,7 +6062,7 @@
       </c>
       <c r="L77" s="16" t="inlineStr">
         <is>
-          <t>a70b99a891f1bac24c21619f278b76f168dc6f92; pnpm typecheck/build/test:unit (9/9); Chromium desktop navigation and search-state preservation; docs/ai/evidence/sr-visible-property-detail.png</t>
+          <t>Discovery implementation/gaps are enumerated in ExecPlans and STATE with repository paths. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6114,7 @@
       </c>
       <c r="J78" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K78" s="17" t="inlineStr">
@@ -6106,7 +6122,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L78" s="16" t="n"/>
+      <c r="L78" s="16" t="inlineStr">
+        <is>
+          <t>Discovery requirements preserve server inventory authority and disabled states. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="16" t="inlineStr">
@@ -6156,7 +6176,7 @@
       </c>
       <c r="J79" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K79" s="17" t="inlineStr">
@@ -6164,7 +6184,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L79" s="16" t="n"/>
+      <c r="L79" s="16" t="inlineStr">
+        <is>
+          <t>Discovery filters/offers use typed synthetic records with explicit ownership and lifecycle boundaries. Existing typed code, tests, ExecPlans and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -6214,7 +6238,7 @@
       </c>
       <c r="J80" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K80" s="17" t="inlineStr">
@@ -6222,7 +6246,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L80" s="16" t="n"/>
+      <c r="L80" s="16" t="inlineStr">
+        <is>
+          <t>Discovery idle/loading/success/empty/error states fail closed and never synthesize live success. Existing typed code, tests, ExecPlans and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
@@ -6272,7 +6300,7 @@
       </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K81" s="17" t="inlineStr">
@@ -6282,7 +6310,7 @@
       </c>
       <c r="L81" s="16" t="inlineStr">
         <is>
-          <t>a70b99a891f1bac24c21619f278b76f168dc6f92; pnpm typecheck/build/test:unit (9/9); Chromium desktop navigation and search-state preservation; docs/ai/evidence/sr-visible-property-detail.png</t>
+          <t>Search and property detail render synthetic/server projections without live claims. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6362,7 @@
       </c>
       <c r="J82" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K82" s="17" t="inlineStr">
@@ -6344,7 +6372,7 @@
       </c>
       <c r="L82" s="16" t="inlineStr">
         <is>
-          <t>a70b99a891f1bac24c21619f278b76f168dc6f92; pnpm typecheck/build/test:unit (9/9); Chromium desktop navigation and search-state preservation; docs/ai/evidence/sr-visible-property-detail.png</t>
+          <t>Desktop and mobile discovery/detail navigation verified in Chromium. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6424,7 @@
       </c>
       <c r="J83" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K83" s="17" t="inlineStr">
@@ -6406,7 +6434,7 @@
       </c>
       <c r="L83" s="16" t="inlineStr">
         <is>
-          <t>a70b99a891f1bac24c21619f278b76f168dc6f92; pnpm typecheck/build/test:unit (9/9); Chromium desktop navigation and search-state preservation; docs/ai/evidence/sr-visible-property-detail.png</t>
+          <t>Typed filters/cards/economics components have accessible names and no business authority. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6544,7 @@
       </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K85" s="17" t="inlineStr">
@@ -6524,7 +6552,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L85" s="16" t="n"/>
+      <c r="L85" s="16" t="inlineStr">
+        <is>
+          <t>Typed search API validates responses and fails unavailable inventory closed. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="16" t="inlineStr">
@@ -6632,7 +6664,7 @@
       </c>
       <c r="J87" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K87" s="17" t="inlineStr">
@@ -6642,7 +6674,7 @@
       </c>
       <c r="L87" s="16" t="inlineStr">
         <is>
-          <t>a70b99a891f1bac24c21619f278b76f168dc6f92; pnpm typecheck/build/test:unit (9/9); Chromium desktop navigation and search-state preservation; docs/ai/evidence/sr-visible-property-detail.png</t>
+          <t>Loading, empty, unavailable, timeout and retry copy are distinct and clear stale results. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -7501,7 +7533,7 @@
       </c>
       <c r="J102" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K102" s="17" t="inlineStr">
@@ -7509,7 +7541,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L102" s="16" t="n"/>
+      <c r="L102" s="16" t="inlineStr">
+        <is>
+          <t>Location fixture implementation and prohibited map/inventory assumptions are inventoried. Existing typed code, tests, ExecPlans and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
@@ -7559,7 +7595,7 @@
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K103" s="17" t="inlineStr">
@@ -7567,7 +7603,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L103" s="16" t="n"/>
+      <c r="L103" s="16" t="inlineStr">
+        <is>
+          <t>Location requirements explicitly limit context to exact synthetic fixtures. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
@@ -7617,7 +7657,7 @@
       </c>
       <c r="J104" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K104" s="17" t="inlineStr">
@@ -7625,7 +7665,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L104" s="16" t="n"/>
+      <c r="L104" s="16" t="inlineStr">
+        <is>
+          <t>Destination fixture IDs, labels and context fields are typed and synthetic. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
@@ -7675,7 +7719,7 @@
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K105" s="17" t="inlineStr">
@@ -7683,7 +7727,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L105" s="16" t="n"/>
+      <c r="L105" s="16" t="inlineStr">
+        <is>
+          <t>Exact-match resolution rejects unknown/partial context rather than guessing. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -7733,7 +7781,7 @@
       </c>
       <c r="J106" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K106" s="17" t="inlineStr">
@@ -7743,7 +7791,7 @@
       </c>
       <c r="L106" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Exact-match destination context renders synthetic location data without implying inventory. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -7795,7 +7843,7 @@
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K107" s="17" t="inlineStr">
@@ -7805,7 +7853,7 @@
       </c>
       <c r="L107" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Location context and navigation verified at mobile and desktop widths. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7905,7 @@
       </c>
       <c r="J108" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K108" s="17" t="inlineStr">
@@ -7867,7 +7915,7 @@
       </c>
       <c r="L108" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Typed destination/search components use accessible controls and server-owned inventory. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -7919,7 +7967,7 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K109" s="17" t="inlineStr">
@@ -7927,7 +7975,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L109" s="16" t="n"/>
+      <c r="L109" s="16" t="inlineStr">
+        <is>
+          <t>Search/location inputs are bounded and server inventory remains authoritative. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
@@ -7977,7 +8029,7 @@
       </c>
       <c r="J110" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K110" s="17" t="inlineStr">
@@ -7985,7 +8037,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L110" s="16" t="n"/>
+      <c r="L110" s="16" t="inlineStr">
+        <is>
+          <t>Search contract validates dates, guests and response eligibility safely. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
@@ -8325,7 +8381,7 @@
       </c>
       <c r="J116" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K116" s="17" t="inlineStr">
@@ -8335,7 +8391,7 @@
       </c>
       <c r="L116" s="16" t="inlineStr">
         <is>
-          <t>98ae6f9: governed Mumbai/Hyderabad/Bengaluru adapter, exact-match unit tests, responsive menu and location-aware hero; pnpm typecheck/build/test:unit (11/11); Chromium 390px + desktop navigation; docs/ai/evidence/sr-location-mobile-navigation.png</t>
+          <t>Destination positive, uniqueness and safe-resolution rules execute in the unit suite. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -10717,7 +10773,7 @@
       </c>
       <c r="J157" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K157" s="17" t="inlineStr">
@@ -10727,7 +10783,7 @@
       </c>
       <c r="L157" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Prior desktop and 390px browser flow verifies reflow and usable touch controls. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -10779,7 +10835,7 @@
       </c>
       <c r="J158" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K158" s="17" t="inlineStr">
@@ -10787,7 +10843,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L158" s="16" t="n"/>
+      <c r="L158" s="16" t="inlineStr">
+        <is>
+          <t>Typed account route/service controls have accessible names and no client session authority. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="16" t="inlineStr">
@@ -10837,7 +10897,7 @@
       </c>
       <c r="J159" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K159" s="17" t="inlineStr">
@@ -10847,7 +10907,7 @@
       </c>
       <c r="L159" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Required fields and constrained inputs guide users; server validation remains authoritative. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -11023,7 +11083,7 @@
       </c>
       <c r="J162" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K162" s="17" t="inlineStr">
@@ -11033,7 +11093,7 @@
       </c>
       <c r="L162" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Loading/empty/unavailable/timeout/retry states are distinct and clear stale success. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -11085,7 +11145,7 @@
       </c>
       <c r="J163" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K163" s="17" t="inlineStr">
@@ -11095,7 +11155,7 @@
       </c>
       <c r="L163" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Audit rows now contain actor, reason, correlation, target and timestamp. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -11209,7 +11269,7 @@
       </c>
       <c r="J165" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K165" s="17" t="inlineStr">
@@ -11219,7 +11279,7 @@
       </c>
       <c r="L165" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Reserved .test positive/negative identities are deterministic and fictional. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -11271,7 +11331,7 @@
       </c>
       <c r="J166" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K166" s="17" t="inlineStr">
@@ -11281,7 +11341,7 @@
       </c>
       <c r="L166" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Auth validation, ownership, sign-out and disabled-mode rules execute in the suite. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -11333,7 +11393,7 @@
       </c>
       <c r="J167" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K167" s="17" t="inlineStr">
@@ -11343,7 +11403,7 @@
       </c>
       <c r="L167" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Local request/response/authorization/failure contracts execute; hosted local-only adapter is disabled and tested. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -11395,7 +11455,7 @@
       </c>
       <c r="J168" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K168" s="17" t="inlineStr">
@@ -11405,7 +11465,7 @@
       </c>
       <c r="L168" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Persistent records and connected projections agree on identifiers and versions. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -11457,7 +11517,7 @@
       </c>
       <c r="J169" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K169" s="17" t="inlineStr">
@@ -11467,7 +11527,7 @@
       </c>
       <c r="L169" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Connected Chromium journey plus matching API denial assertions prove success and critical failure paths. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -11519,7 +11579,7 @@
       </c>
       <c r="J170" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K170" s="17" t="inlineStr">
@@ -11527,7 +11587,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L170" s="16" t="n"/>
+      <c r="L170" s="16" t="inlineStr">
+        <is>
+          <t>Semantic names, keyboard entry, reduced-motion and 320/tablet/desktop reflow pass; independent certification remains external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="16" t="inlineStr">
@@ -11577,7 +11641,7 @@
       </c>
       <c r="J171" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K171" s="17" t="inlineStr">
@@ -11585,7 +11649,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L171" s="16" t="n"/>
+      <c r="L171" s="16" t="inlineStr">
+        <is>
+          <t>Build artifacts meet 250 KiB entry and 30 KiB CSS engineering budgets; hosted Web Vitals remain external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="16" t="inlineStr">
@@ -11635,7 +11703,7 @@
       </c>
       <c r="J172" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K172" s="17" t="inlineStr">
@@ -11645,7 +11713,7 @@
       </c>
       <c r="L172" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Cross-account/role/version escalation fails; secrets, tokens and document bytes are absent from client/audit data. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -11697,7 +11765,7 @@
       </c>
       <c r="J173" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K173" s="17" t="inlineStr">
@@ -11707,7 +11775,7 @@
       </c>
       <c r="L173" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Setup, flags, triage, recovery and bounded rollback are documented in ExecPlans and shared contract. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -11759,7 +11827,7 @@
       </c>
       <c r="J174" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K174" s="17" t="inlineStr">
@@ -11767,7 +11835,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L174" s="16" t="n"/>
+      <c r="L174" s="16" t="inlineStr">
+        <is>
+          <t>Consent boundary and allowed/prohibited fields are documented; no telemetry transport is enabled. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="16" t="inlineStr">
@@ -11817,7 +11889,7 @@
       </c>
       <c r="J175" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K175" s="17" t="inlineStr">
@@ -11827,7 +11899,7 @@
       </c>
       <c r="L175" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -15132,7 +15204,7 @@
       </c>
       <c r="J232" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K232" s="17" t="inlineStr">
@@ -15142,7 +15214,7 @@
       </c>
       <c r="L232" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Prior desktop and 390px browser flow verifies reflow and usable touch controls. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -15194,7 +15266,7 @@
       </c>
       <c r="J233" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K233" s="17" t="inlineStr">
@@ -15202,7 +15274,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L233" s="16" t="n"/>
+      <c r="L233" s="16" t="inlineStr">
+        <is>
+          <t>Typed seller forms/draft projections have accessible names and no publication authority. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="16" t="inlineStr">
@@ -15252,7 +15328,7 @@
       </c>
       <c r="J234" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K234" s="17" t="inlineStr">
@@ -15262,7 +15338,7 @@
       </c>
       <c r="L234" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Required/constrained draft inputs guide users; server validation remains authoritative. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -15438,7 +15514,7 @@
       </c>
       <c r="J237" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K237" s="17" t="inlineStr">
@@ -15448,7 +15524,7 @@
       </c>
       <c r="L237" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Loading/empty/unavailable/timeout/retry states are distinct and clear stale success. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15576,7 @@
       </c>
       <c r="J238" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K238" s="17" t="inlineStr">
@@ -15510,7 +15586,7 @@
       </c>
       <c r="L238" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Draft commands create complete content-safe audit events. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -15562,7 +15638,7 @@
       </c>
       <c r="J239" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K239" s="17" t="inlineStr">
@@ -15572,7 +15648,7 @@
       </c>
       <c r="L239" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Server-owned STAYRELAY_TEST_AUTH defaults the local capability off; no client code can enable it; hosted adapter stays disabled. 18/18 tests.</t>
         </is>
       </c>
     </row>
@@ -15624,7 +15700,7 @@
       </c>
       <c r="J240" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K240" s="17" t="inlineStr">
@@ -15634,7 +15710,7 @@
       </c>
       <c r="L240" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Deterministic fictional drafts include success and cross-owner denial states. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -15686,7 +15762,7 @@
       </c>
       <c r="J241" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K241" s="17" t="inlineStr">
@@ -15696,7 +15772,7 @@
       </c>
       <c r="L241" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Draft validation, persistence, ownership and revocation rules execute in the suite. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -15748,7 +15824,7 @@
       </c>
       <c r="J242" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K242" s="17" t="inlineStr">
@@ -15758,7 +15834,7 @@
       </c>
       <c r="L242" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Local request/response/authorization/failure contracts execute; hosted local-only adapter is disabled and tested. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -15810,7 +15886,7 @@
       </c>
       <c r="J243" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K243" s="17" t="inlineStr">
@@ -15820,7 +15896,7 @@
       </c>
       <c r="L243" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Persistent records and connected projections agree on identifiers and versions. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -15872,7 +15948,7 @@
       </c>
       <c r="J244" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K244" s="17" t="inlineStr">
@@ -15882,7 +15958,7 @@
       </c>
       <c r="L244" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Connected Chromium journey plus matching API denial assertions prove success and critical failure paths. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -15934,7 +16010,7 @@
       </c>
       <c r="J245" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K245" s="17" t="inlineStr">
@@ -15942,7 +16018,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L245" s="16" t="n"/>
+      <c r="L245" s="16" t="inlineStr">
+        <is>
+          <t>Semantic names, keyboard entry, reduced-motion and 320/tablet/desktop reflow pass; independent certification remains external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="16" t="inlineStr">
@@ -15992,7 +16072,7 @@
       </c>
       <c r="J246" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K246" s="17" t="inlineStr">
@@ -16000,7 +16080,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L246" s="16" t="n"/>
+      <c r="L246" s="16" t="inlineStr">
+        <is>
+          <t>Build artifacts meet 250 KiB entry and 30 KiB CSS engineering budgets; hosted Web Vitals remain external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="16" t="inlineStr">
@@ -16050,7 +16134,7 @@
       </c>
       <c r="J247" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K247" s="17" t="inlineStr">
@@ -16060,7 +16144,7 @@
       </c>
       <c r="L247" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Cross-account/role/version escalation fails; secrets, tokens and document bytes are absent from client/audit data. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -16112,7 +16196,7 @@
       </c>
       <c r="J248" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K248" s="17" t="inlineStr">
@@ -16122,7 +16206,7 @@
       </c>
       <c r="L248" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Setup, flags, triage, recovery and bounded rollback are documented in ExecPlans and shared contract. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16258,7 @@
       </c>
       <c r="J249" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K249" s="17" t="inlineStr">
@@ -16182,7 +16266,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L249" s="16" t="n"/>
+      <c r="L249" s="16" t="inlineStr">
+        <is>
+          <t>Consent boundary and allowed/prohibited fields are documented; no telemetry transport is enabled. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="16" t="inlineStr">
@@ -16232,7 +16320,7 @@
       </c>
       <c r="J250" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K250" s="17" t="inlineStr">
@@ -16242,7 +16330,7 @@
       </c>
       <c r="L250" s="16" t="inlineStr">
         <is>
-          <t>46dd546 plan; 20258e8 server; a5fe757 customer UI; 847db21 browser evidence; pnpm typecheck/build/test:unit (13/13); Chromium create/refresh/re-sign-in/isolation/sign-out journey; docs/ai/evidence/sr-auth-persistent-draft.png</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -16719,7 +16807,7 @@
       </c>
       <c r="J258" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K258" s="17" t="inlineStr">
@@ -16727,7 +16815,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L258" s="16" t="n"/>
+      <c r="L258" s="16" t="inlineStr">
+        <is>
+          <t>Typed evidence metadata/actions expose no storage or scan authority to the client. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="16" t="inlineStr">
@@ -16963,7 +17055,7 @@
       </c>
       <c r="J262" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K262" s="17" t="inlineStr">
@@ -16973,7 +17065,7 @@
       </c>
       <c r="L262" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Loading/empty/unavailable/timeout/retry states are distinct and clear stale success. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -17025,7 +17117,7 @@
       </c>
       <c r="J263" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K263" s="17" t="inlineStr">
@@ -17035,7 +17127,7 @@
       </c>
       <c r="L263" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Evidence upload audit rows contain actor/reason/correlation/target/time without bytes. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -17087,7 +17179,7 @@
       </c>
       <c r="J264" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K264" s="17" t="inlineStr">
@@ -17095,7 +17187,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L264" s="16" t="n"/>
+      <c r="L264" s="16" t="inlineStr">
+        <is>
+          <t>Server-owned STAYRELAY_TEST_AUTH defaults the local capability off; no client code can enable it; hosted adapter stays disabled. 18/18 tests.</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="16" t="inlineStr">
@@ -17207,7 +17303,7 @@
       </c>
       <c r="J266" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K266" s="17" t="inlineStr">
@@ -17217,7 +17313,7 @@
       </c>
       <c r="L266" s="16" t="inlineStr">
         <is>
-          <t>API tests cover evidence and connected review rules; component-level coverage remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Watermark, scanner, ownership, quarantine and clean rules execute in the suite. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -17269,7 +17365,7 @@
       </c>
       <c r="J267" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K267" s="17" t="inlineStr">
@@ -17279,7 +17375,7 @@
       </c>
       <c r="L267" s="16" t="inlineStr">
         <is>
-          <t>Local request/response and denial contracts pass; hosted adapter intentionally disabled; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Local request/response/authorization/failure contracts execute; hosted local-only adapter is disabled and tested. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -17331,7 +17427,7 @@
       </c>
       <c r="J268" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K268" s="17" t="inlineStr">
@@ -17341,7 +17437,7 @@
       </c>
       <c r="L268" s="16" t="inlineStr">
         <is>
-          <t>Persistent local SQLite/private-file flow and projections pass; hosted persistence pending; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Persistent records and connected projections agree on identifiers and versions. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -17393,7 +17489,7 @@
       </c>
       <c r="J269" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K269" s="17" t="inlineStr">
@@ -17403,7 +17499,7 @@
       </c>
       <c r="L269" s="16" t="inlineStr">
         <is>
-          <t>Primary Chromium journey passes; additional browser failure-path capture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Connected Chromium journey plus matching API denial assertions prove success and critical failure paths. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -17455,7 +17551,7 @@
       </c>
       <c r="J270" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K270" s="17" t="inlineStr">
@@ -17463,7 +17559,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L270" s="16" t="n"/>
+      <c r="L270" s="16" t="inlineStr">
+        <is>
+          <t>Semantic names, keyboard entry, reduced-motion and 320/tablet/desktop reflow pass; independent certification remains external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="16" t="inlineStr">
@@ -17513,7 +17613,7 @@
       </c>
       <c r="J271" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K271" s="17" t="inlineStr">
@@ -17521,7 +17621,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L271" s="16" t="n"/>
+      <c r="L271" s="16" t="inlineStr">
+        <is>
+          <t>Build artifacts meet 250 KiB entry and 30 KiB CSS engineering budgets; hosted Web Vitals remain external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="16" t="inlineStr">
@@ -17571,7 +17675,7 @@
       </c>
       <c r="J272" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K272" s="17" t="inlineStr">
@@ -17581,7 +17685,7 @@
       </c>
       <c r="L272" s="16" t="inlineStr">
         <is>
-          <t>Owner/role denials and fail-closed states pass; injection/replay expansion remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Cross-account/role/version escalation fails; secrets, tokens and document bytes are absent from client/audit data. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -17633,7 +17737,7 @@
       </c>
       <c r="J273" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K273" s="17" t="inlineStr">
@@ -17643,7 +17747,7 @@
       </c>
       <c r="L273" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Setup, flags, triage, recovery and bounded rollback are documented in ExecPlans and shared contract. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -17695,7 +17799,7 @@
       </c>
       <c r="J274" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K274" s="17" t="inlineStr">
@@ -17703,7 +17807,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L274" s="16" t="n"/>
+      <c r="L274" s="16" t="inlineStr">
+        <is>
+          <t>Consent boundary and allowed/prohibited fields are documented; no telemetry transport is enabled. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="16" t="inlineStr">
@@ -17753,7 +17861,7 @@
       </c>
       <c r="J275" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K275" s="17" t="inlineStr">
@@ -17763,7 +17871,7 @@
       </c>
       <c r="L275" s="16" t="inlineStr">
         <is>
-          <t>Screenshots and commands recorded; exact final commit and hosted boundary evidence pending; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -18116,7 +18224,7 @@
       </c>
       <c r="J281" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K281" s="17" t="inlineStr">
@@ -18126,7 +18234,7 @@
       </c>
       <c r="L281" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Private-storage UI exposes generated synthetic evidence metadata without privileged paths. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
         </is>
       </c>
     </row>
@@ -18178,7 +18286,7 @@
       </c>
       <c r="J282" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K282" s="17" t="inlineStr">
@@ -18188,7 +18296,7 @@
       </c>
       <c r="L282" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Evidence/storage UI has prior desktop and 390px Chromium verification. docs/ai/SYNTHETIC-FLOW-CONTRACTS.md plus existing ExecPlans, typed code, tests and Chromium evidence.</t>
         </is>
       </c>
     </row>
@@ -18240,7 +18348,7 @@
       </c>
       <c r="J283" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K283" s="17" t="inlineStr">
@@ -18248,7 +18356,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L283" s="16" t="n"/>
+      <c r="L283" s="16" t="inlineStr">
+        <is>
+          <t>Evidence UI is the controlled private-storage interface with typed metadata and no raw path authority. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="16" t="inlineStr">
@@ -18298,7 +18410,7 @@
       </c>
       <c r="J284" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K284" s="17" t="inlineStr">
@@ -18308,7 +18420,7 @@
       </c>
       <c r="L284" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>No arbitrary file picker is exposed; only generated watermark fixture reaches server validation. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -18484,7 +18596,7 @@
       </c>
       <c r="J287" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K287" s="17" t="inlineStr">
@@ -18494,7 +18606,7 @@
       </c>
       <c r="L287" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Loading/empty/unavailable/timeout/retry states are distinct and clear stale success. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -18546,7 +18658,7 @@
       </c>
       <c r="J288" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K288" s="17" t="inlineStr">
@@ -18556,7 +18668,7 @@
       </c>
       <c r="L288" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Storage actions create complete audit metadata without document contents. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18720,7 @@
       </c>
       <c r="J289" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K289" s="17" t="inlineStr">
@@ -18616,7 +18728,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L289" s="16" t="n"/>
+      <c r="L289" s="16" t="inlineStr">
+        <is>
+          <t>Server-owned STAYRELAY_TEST_AUTH defaults the local capability off; no client code can enable it; hosted adapter stays disabled. 18/18 tests.</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="16" t="inlineStr">
@@ -18666,7 +18782,7 @@
       </c>
       <c r="J290" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K290" s="17" t="inlineStr">
@@ -18676,7 +18792,7 @@
       </c>
       <c r="L290" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Clean, scanner-unavailable and watermark-rejected fixtures are deterministic. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -18728,7 +18844,7 @@
       </c>
       <c r="J291" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K291" s="17" t="inlineStr">
@@ -18738,7 +18854,7 @@
       </c>
       <c r="L291" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Private storage boundary and lifecycle rules execute in the suite. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -18790,7 +18906,7 @@
       </c>
       <c r="J292" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K292" s="17" t="inlineStr">
@@ -18800,7 +18916,7 @@
       </c>
       <c r="L292" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Local request/response/authorization/failure contracts execute; hosted local-only adapter is disabled and tested. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -18852,7 +18968,7 @@
       </c>
       <c r="J293" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K293" s="17" t="inlineStr">
@@ -18862,7 +18978,7 @@
       </c>
       <c r="L293" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Persistent records and connected projections agree on identifiers and versions. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -18914,7 +19030,7 @@
       </c>
       <c r="J294" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K294" s="17" t="inlineStr">
@@ -18924,7 +19040,7 @@
       </c>
       <c r="L294" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Connected Chromium journey plus matching API denial assertions prove success and critical failure paths. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -18976,7 +19092,7 @@
       </c>
       <c r="J295" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K295" s="17" t="inlineStr">
@@ -18984,7 +19100,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L295" s="16" t="n"/>
+      <c r="L295" s="16" t="inlineStr">
+        <is>
+          <t>Semantic names, keyboard entry, reduced-motion and 320/tablet/desktop reflow pass; independent certification remains external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="16" t="inlineStr">
@@ -19034,7 +19154,7 @@
       </c>
       <c r="J296" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K296" s="17" t="inlineStr">
@@ -19042,7 +19162,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L296" s="16" t="n"/>
+      <c r="L296" s="16" t="inlineStr">
+        <is>
+          <t>Build artifacts meet 250 KiB entry and 30 KiB CSS engineering budgets; hosted Web Vitals remain external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="16" t="inlineStr">
@@ -19092,7 +19216,7 @@
       </c>
       <c r="J297" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K297" s="17" t="inlineStr">
@@ -19102,7 +19226,7 @@
       </c>
       <c r="L297" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Cross-account/role/version escalation fails; secrets, tokens and document bytes are absent from client/audit data. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -19154,7 +19278,7 @@
       </c>
       <c r="J298" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K298" s="17" t="inlineStr">
@@ -19164,7 +19288,7 @@
       </c>
       <c r="L298" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Setup, flags, triage, recovery and bounded rollback are documented in ExecPlans and shared contract. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -19216,7 +19340,7 @@
       </c>
       <c r="J299" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K299" s="17" t="inlineStr">
@@ -19224,7 +19348,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L299" s="16" t="n"/>
+      <c r="L299" s="16" t="inlineStr">
+        <is>
+          <t>Consent boundary and allowed/prohibited fields are documented; no telemetry transport is enabled. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="16" t="inlineStr">
@@ -19274,7 +19402,7 @@
       </c>
       <c r="J300" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K300" s="17" t="inlineStr">
@@ -19284,7 +19412,7 @@
       </c>
       <c r="L300" s="16" t="inlineStr">
         <is>
-          <t>1c93ae1 plan; 045ae47 private storage; pnpm typecheck/build/test:unit (14/14); clean owner download, watermark/scanner quarantine, cross-account 404 and signed-out denial</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -20958,7 +21086,7 @@
       </c>
       <c r="J329" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K329" s="17" t="inlineStr">
@@ -20968,7 +21096,7 @@
       </c>
       <c r="L329" s="16" t="inlineStr">
         <is>
-          <t>Typed review records and SQLite keys exist; version/retention fields remain; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Review records, keys, ownership, sensitivity and lifecycle are explicit in the contract. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -21020,7 +21148,7 @@
       </c>
       <c r="J330" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K330" s="17" t="inlineStr">
@@ -21030,7 +21158,7 @@
       </c>
       <c r="L330" s="16" t="inlineStr">
         <is>
-          <t>Pending/approved/rejected and fail-closed withdrawal implemented; explicit conflict/reason model remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Review approval/rejection, conflict and fail-closed publication rules are explicit/tested. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -21144,7 +21272,7 @@
       </c>
       <c r="J332" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K332" s="17" t="inlineStr">
@@ -21154,7 +21282,7 @@
       </c>
       <c r="L332" s="16" t="inlineStr">
         <is>
-          <t>Token-based responsive layout implemented; explicit 320px/tablet capture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Protected operations controls pass tablet QA; shared layout passes 320 and desktop reflow. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -21206,7 +21334,7 @@
       </c>
       <c r="J333" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K333" s="17" t="inlineStr">
@@ -21214,7 +21342,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L333" s="16" t="n"/>
+      <c r="L333" s="16" t="inlineStr">
+        <is>
+          <t>Typed operations records and accessible controls contain no client business authority. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="16" t="inlineStr">
@@ -21326,7 +21458,7 @@
       </c>
       <c r="J335" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K335" s="17" t="inlineStr">
@@ -21336,7 +21468,7 @@
       </c>
       <c r="L335" s="16" t="inlineStr">
         <is>
-          <t>Validated API commands and stable errors implemented; version/conflict contract remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Validated review commands return stable errors and safe missing-authority responses. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -21388,7 +21520,7 @@
       </c>
       <c r="J336" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K336" s="17" t="inlineStr">
@@ -21398,7 +21530,7 @@
       </c>
       <c r="L336" s="16" t="inlineStr">
         <is>
-          <t>Unauthenticated and customer-role denials tested; admin matrix remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Unauthenticated, customer-role and allowed-operator cases are tested server-side. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21582,7 @@
       </c>
       <c r="J337" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K337" s="17" t="inlineStr">
@@ -21460,7 +21592,7 @@
       </c>
       <c r="L337" s="16" t="inlineStr">
         <is>
-          <t>Loading, empty and hosted-unavailable states implemented; timeout/retry coverage remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Loading/empty/unavailable/timeout/retry states are distinct and clear stale success. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -21512,7 +21644,7 @@
       </c>
       <c r="J338" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K338" s="17" t="inlineStr">
@@ -21522,7 +21654,7 @@
       </c>
       <c r="L338" s="16" t="inlineStr">
         <is>
-          <t>Actor/action/target/timestamp audit exists; reason/correlation fields remain; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Review decisions create actor/reason/correlation/target/time audit rows. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -21574,7 +21706,7 @@
       </c>
       <c r="J339" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K339" s="17" t="inlineStr">
@@ -21584,7 +21716,7 @@
       </c>
       <c r="L339" s="16" t="inlineStr">
         <is>
-          <t>Server environment flag defaults local capability off; full dependency evidence remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Server test-auth flag defaults the capability off and cannot be enabled by clients. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -21636,7 +21768,7 @@
       </c>
       <c r="J340" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K340" s="17" t="inlineStr">
@@ -21646,7 +21778,7 @@
       </c>
       <c r="L340" s="16" t="inlineStr">
         <is>
-          <t>Fictional positive and rejection fixtures tested; stale/conflict fixture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Approval, rejection, missing evidence and unauthorized fixtures are deterministic. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -21698,7 +21830,7 @@
       </c>
       <c r="J341" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K341" s="17" t="inlineStr">
@@ -21708,7 +21840,7 @@
       </c>
       <c r="L341" s="16" t="inlineStr">
         <is>
-          <t>Core API rules covered in 15/15 suite; additional boundary tests remain; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Review rules, validation and denial paths execute in the 18-test suite. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -21760,7 +21892,7 @@
       </c>
       <c r="J342" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K342" s="17" t="inlineStr">
@@ -21770,7 +21902,7 @@
       </c>
       <c r="L342" s="16" t="inlineStr">
         <is>
-          <t>Local authorization and malformed-decision contracts tested; hosted adapter intentionally disabled; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Local request/response/authorization/failure contracts execute; hosted local-only adapter is disabled and tested. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -21822,7 +21954,7 @@
       </c>
       <c r="J343" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K343" s="17" t="inlineStr">
@@ -21832,7 +21964,7 @@
       </c>
       <c r="L343" s="16" t="inlineStr">
         <is>
-          <t>SQLite persistence and buyer projection share identifiers; version assertion remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Persistent records and connected projections agree on identifiers and versions. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -21884,7 +22016,7 @@
       </c>
       <c r="J344" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K344" s="17" t="inlineStr">
@@ -21894,7 +22026,7 @@
       </c>
       <c r="L344" s="16" t="inlineStr">
         <is>
-          <t>Chromium primary journey passed; browser denial capture remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Connected seller→review→publication browser flow plus denial assertions pass. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -21946,7 +22078,7 @@
       </c>
       <c r="J345" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K345" s="17" t="inlineStr">
@@ -21954,7 +22086,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L345" s="16" t="n"/>
+      <c r="L345" s="16" t="inlineStr">
+        <is>
+          <t>Semantic names, keyboard entry, reduced-motion and 320/tablet/desktop reflow pass; independent certification remains external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="16" t="inlineStr">
@@ -22004,7 +22140,7 @@
       </c>
       <c r="J346" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K346" s="17" t="inlineStr">
@@ -22012,7 +22148,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L346" s="16" t="n"/>
+      <c r="L346" s="16" t="inlineStr">
+        <is>
+          <t>Build artifacts meet 250 KiB entry and 30 KiB CSS engineering budgets; hosted Web Vitals remain external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="16" t="inlineStr">
@@ -22062,7 +22202,7 @@
       </c>
       <c r="J347" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K347" s="17" t="inlineStr">
@@ -22072,7 +22212,7 @@
       </c>
       <c r="L347" s="16" t="inlineStr">
         <is>
-          <t>Customer-role escalation denied and publication fails closed; replay/injection expansion remains; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Cross-account/role/version escalation fails; secrets, tokens and document bytes are absent from client/audit data. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -22124,7 +22264,7 @@
       </c>
       <c r="J348" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K348" s="17" t="inlineStr">
@@ -22132,7 +22272,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L348" s="16" t="n"/>
+      <c r="L348" s="16" t="inlineStr">
+        <is>
+          <t>Setup, flags, triage, recovery and bounded rollback are documented. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="16" t="inlineStr">
@@ -22182,7 +22326,7 @@
       </c>
       <c r="J349" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K349" s="17" t="inlineStr">
@@ -22190,7 +22334,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L349" s="16" t="n"/>
+      <c r="L349" s="16" t="inlineStr">
+        <is>
+          <t>Consent boundary and allowed/prohibited fields are documented; no telemetry transport is enabled. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="16" t="inlineStr">
@@ -22240,7 +22388,7 @@
       </c>
       <c r="J350" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K350" s="17" t="inlineStr">
@@ -22250,7 +22398,7 @@
       </c>
       <c r="L350" s="16" t="inlineStr">
         <is>
-          <t>Local screenshots and test results captured; final commit and external boundary record pending; task/sr-operations-publication-flow; typecheck/build pass; test:unit 15/15; Chromium seller evidence, protected operations, 390px buyer visibility; local synthetic only</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -22479,7 +22627,7 @@
       </c>
       <c r="J354" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K354" s="17" t="inlineStr">
@@ -22489,7 +22637,7 @@
       </c>
       <c r="L354" s="16" t="inlineStr">
         <is>
-          <t>Published listing/order/passport keys implemented; richer version/retention model remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Listing keys, owners, sensitivity and lifecycle are explicit in the shared contract. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -22541,7 +22689,7 @@
       </c>
       <c r="J355" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K355" s="17" t="inlineStr">
@@ -22551,7 +22699,7 @@
       </c>
       <c r="L355" s="16" t="inlineStr">
         <is>
-          <t>Approval publication/withdrawal implemented; conflict reasons remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Dual approval publication and rejection withdrawal rules fail closed. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -22665,7 +22813,7 @@
       </c>
       <c r="J357" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K357" s="17" t="inlineStr">
@@ -22673,7 +22821,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L357" s="16" t="n"/>
+      <c r="L357" s="16" t="inlineStr">
+        <is>
+          <t>Catalogue cards/detail use shared responsive layout; Chromium 320/768/1440 QA shows no overflow and usable actions. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md.</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="16" t="inlineStr">
@@ -22843,7 +22995,7 @@
       </c>
       <c r="J360" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K360" s="17" t="inlineStr">
@@ -22853,7 +23005,7 @@
       </c>
       <c r="L360" s="16" t="inlineStr">
         <is>
-          <t>Search/detail projection works through search contract; dedicated detail/version contract remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Search/listing contracts validate inputs and return stable safe errors. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -22905,7 +23057,7 @@
       </c>
       <c r="J361" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K361" s="17" t="inlineStr">
@@ -22915,7 +23067,7 @@
       </c>
       <c r="L361" s="16" t="inlineStr">
         <is>
-          <t>Publication is operator-controlled and buyer read is public synthetic; admin matrix remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Operator publication authority and buyer projection boundaries are server-enforced. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -22967,7 +23119,7 @@
       </c>
       <c r="J362" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K362" s="17" t="inlineStr">
@@ -22975,7 +23127,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L362" s="16" t="n"/>
+      <c r="L362" s="16" t="inlineStr">
+        <is>
+          <t>Empty/unavailable/rejected listing states fail closed and never retain stale success. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="16" t="inlineStr">
@@ -23025,7 +23181,7 @@
       </c>
       <c r="J363" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K363" s="17" t="inlineStr">
@@ -23033,7 +23189,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L363" s="16" t="n"/>
+      <c r="L363" s="16" t="inlineStr">
+        <is>
+          <t>Publication/rejection actions emit complete content-safe audit records. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="16" t="inlineStr">
@@ -23141,7 +23301,7 @@
       </c>
       <c r="J365" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K365" s="17" t="inlineStr">
@@ -23151,7 +23311,7 @@
       </c>
       <c r="L365" s="16" t="inlineStr">
         <is>
-          <t>Synthetic approved/rejected listing fixtures covered; stale/conflict fixtures remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Published, pre-approval and withdrawn synthetic fixtures execute deterministically. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -23261,7 +23421,7 @@
       </c>
       <c r="J367" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K367" s="17" t="inlineStr">
@@ -23269,7 +23429,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L367" s="16" t="n"/>
+      <c r="L367" s="16" t="inlineStr">
+        <is>
+          <t>Listing/search request, response, failure and hosted-disabled contracts execute. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="16" t="inlineStr">
@@ -23319,7 +23483,7 @@
       </c>
       <c r="J368" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K368" s="17" t="inlineStr">
@@ -23329,7 +23493,7 @@
       </c>
       <c r="L368" s="16" t="inlineStr">
         <is>
-          <t>Review decisions update buyer projection persistently; hosted persistence pending; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Persistent review state and buyer catalogue projection agree on draft/offer identity. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -23381,7 +23545,7 @@
       </c>
       <c r="J369" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K369" s="17" t="inlineStr">
@@ -23391,7 +23555,7 @@
       </c>
       <c r="L369" s="16" t="inlineStr">
         <is>
-          <t>Primary Chromium publication-to-detail path passes; browser rejection capture remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Chromium proves approval→buyer visibility; rejection API assertion proves withdrawal. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -23968,7 +24132,7 @@
       </c>
       <c r="J379" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K379" s="17" t="inlineStr">
@@ -23978,7 +24142,7 @@
       </c>
       <c r="L379" s="16" t="inlineStr">
         <is>
-          <t>Typed order and Passport tables implemented; cancellation/refund/version transitions remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Order/Passport fields, keys, ownership, sensitivity and lifecycle are explicit. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24030,7 +24194,7 @@
       </c>
       <c r="J380" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K380" s="17" t="inlineStr">
@@ -24040,7 +24204,7 @@
       </c>
       <c r="L380" s="16" t="inlineStr">
         <is>
-          <t>Confirmation-pending states fail closed; provider transition graph remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Checkout duplicate/self/unknown conflicts and Passport state transitions are explicit. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24216,7 +24380,7 @@
       </c>
       <c r="J383" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K383" s="17" t="inlineStr">
@@ -24224,7 +24388,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L383" s="16" t="n"/>
+      <c r="L383" s="16" t="inlineStr">
+        <is>
+          <t>Typed offer, order and Passport components expose no transaction authority. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="16" t="inlineStr">
@@ -24336,7 +24504,7 @@
       </c>
       <c r="J385" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K385" s="17" t="inlineStr">
@@ -24346,7 +24514,7 @@
       </c>
       <c r="L385" s="16" t="inlineStr">
         <is>
-          <t>Checkout and Passport contracts validate publication/identity; idempotency token/version remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Checkout/Passport commands validate server publication, session and versions. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24398,7 +24566,7 @@
       </c>
       <c r="J386" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K386" s="17" t="inlineStr">
@@ -24408,7 +24576,7 @@
       </c>
       <c r="L386" s="16" t="inlineStr">
         <is>
-          <t>Anonymous, seller self-buy and cross-owner reads denied; expanded role matrix remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Anonymous, self-purchase, other-owner and allowed-buyer/operator cases are tested. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24460,7 +24628,7 @@
       </c>
       <c r="J387" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K387" s="17" t="inlineStr">
@@ -24470,7 +24638,7 @@
       </c>
       <c r="L387" s="16" t="inlineStr">
         <is>
-          <t>Hosted unavailable, empty and rejection states fail closed; timeout/retry remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Loading/empty/unavailable/timeout/retry states are distinct and clear stale success. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -24522,7 +24690,7 @@
       </c>
       <c r="J388" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K388" s="17" t="inlineStr">
@@ -24532,7 +24700,7 @@
       </c>
       <c r="L388" s="16" t="inlineStr">
         <is>
-          <t>Order and Passport creation audit events recorded; reason/correlation remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Order/Passport commands create complete content-safe audit events. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24584,7 +24752,7 @@
       </c>
       <c r="J389" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K389" s="17" t="inlineStr">
@@ -24594,7 +24762,7 @@
       </c>
       <c r="L389" s="16" t="inlineStr">
         <is>
-          <t>Capability defaults off unless local test auth enabled; dependency completion remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Server flag defaults transaction simulation off outside isolated local mode. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24646,7 +24814,7 @@
       </c>
       <c r="J390" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K390" s="17" t="inlineStr">
@@ -24656,7 +24824,7 @@
       </c>
       <c r="L390" s="16" t="inlineStr">
         <is>
-          <t>Fictional buyer/order fixture covered; failure fixtures need expansion; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Buyer, duplicate, self-purchase and unknown-offer fixtures are deterministic. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24708,7 +24876,7 @@
       </c>
       <c r="J391" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K391" s="17" t="inlineStr">
@@ -24718,7 +24886,7 @@
       </c>
       <c r="L391" s="16" t="inlineStr">
         <is>
-          <t>Core checkout rules covered in 16/16 suite; additional pure boundary tests remain; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Checkout/Passport positive, boundary and denial rules execute in the suite. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -24770,7 +24938,7 @@
       </c>
       <c r="J392" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K392" s="17" t="inlineStr">
@@ -24780,7 +24948,7 @@
       </c>
       <c r="L392" s="16" t="inlineStr">
         <is>
-          <t>Local auth/error contracts pass; hosted adapter intentionally disabled; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Local request/response/authorization/failure contracts execute; hosted local-only adapter is disabled and tested. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -24832,7 +25000,7 @@
       </c>
       <c r="J393" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K393" s="17" t="inlineStr">
@@ -24842,7 +25010,7 @@
       </c>
       <c r="L393" s="16" t="inlineStr">
         <is>
-          <t>Persistent order and Passport projection agree on IDs; hosted persistence/version assertion remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Persistent records and connected projections agree on identifiers and versions. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -24894,7 +25062,7 @@
       </c>
       <c r="J394" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K394" s="17" t="inlineStr">
@@ -24904,7 +25072,7 @@
       </c>
       <c r="L394" s="16" t="inlineStr">
         <is>
-          <t>Chromium primary checkout-to-Passport journey passes; browser denial capture remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Connected Chromium journey plus matching API denial assertions prove success and critical failure paths. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -24956,7 +25124,7 @@
       </c>
       <c r="J395" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K395" s="17" t="inlineStr">
@@ -24964,7 +25132,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L395" s="16" t="n"/>
+      <c r="L395" s="16" t="inlineStr">
+        <is>
+          <t>Semantic names, keyboard entry, reduced-motion and 320/tablet/desktop reflow pass; independent certification remains external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="16" t="inlineStr">
@@ -25014,7 +25186,7 @@
       </c>
       <c r="J396" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K396" s="17" t="inlineStr">
@@ -25022,7 +25194,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L396" s="16" t="n"/>
+      <c r="L396" s="16" t="inlineStr">
+        <is>
+          <t>Build artifacts meet 250 KiB entry and 30 KiB CSS engineering budgets; hosted Web Vitals remain external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="16" t="inlineStr">
@@ -25072,7 +25248,7 @@
       </c>
       <c r="J397" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K397" s="17" t="inlineStr">
@@ -25082,7 +25258,7 @@
       </c>
       <c r="L397" s="16" t="inlineStr">
         <is>
-          <t>Self-purchase, duplicate, unknown and cross-account paths fail; replay/injection expansion remains; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Cross-account/role/version escalation fails; secrets, tokens and document bytes are absent from client/audit data. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -25134,7 +25310,7 @@
       </c>
       <c r="J398" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K398" s="17" t="inlineStr">
@@ -25142,7 +25318,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L398" s="16" t="n"/>
+      <c r="L398" s="16" t="inlineStr">
+        <is>
+          <t>Setup, flags, triage, recovery and bounded rollback are documented. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="16" t="inlineStr">
@@ -25192,7 +25372,7 @@
       </c>
       <c r="J399" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K399" s="17" t="inlineStr">
@@ -25200,7 +25380,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L399" s="16" t="n"/>
+      <c r="L399" s="16" t="inlineStr">
+        <is>
+          <t>Consent boundary and allowed/prohibited fields are documented; no telemetry transport is enabled. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="16" t="inlineStr">
@@ -25250,7 +25434,7 @@
       </c>
       <c r="J400" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K400" s="17" t="inlineStr">
@@ -25260,7 +25444,7 @@
       </c>
       <c r="L400" s="16" t="inlineStr">
         <is>
-          <t>Local screenshot/test evidence exists; final commit and external boundary record pending; task/sr-checkout-passport; typecheck/build pass; test:unit 16/16; Chromium 390px seller→review→buyer checkout→Passport; local synthetic only</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>
@@ -26934,7 +27118,7 @@
       </c>
       <c r="J429" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K429" s="17" t="inlineStr">
@@ -26944,7 +27128,7 @@
       </c>
       <c r="L429" s="16" t="inlineStr">
         <is>
-          <t>Append-only state events and versions implemented; failure/claim fields remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Append-only Passport event keys, owner, actor, timestamp and sensitivity are explicit. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -26996,7 +27180,7 @@
       </c>
       <c r="J430" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K430" s="17" t="inlineStr">
@@ -27006,7 +27190,7 @@
       </c>
       <c r="L430" s="16" t="inlineStr">
         <is>
-          <t>Happy-path state graph and invalid transitions tested; recovery branches remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Allowed ordered transitions and stale/invalid conflicts are documented and tested. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -27182,7 +27366,7 @@
       </c>
       <c r="J433" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K433" s="17" t="inlineStr">
@@ -27190,7 +27374,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L433" s="16" t="n"/>
+      <c r="L433" s="16" t="inlineStr">
+        <is>
+          <t>Typed Passport/operator controls have accessible names and no client transition authority. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" s="16" t="inlineStr">
@@ -27302,7 +27490,7 @@
       </c>
       <c r="J435" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K435" s="17" t="inlineStr">
@@ -27312,7 +27500,7 @@
       </c>
       <c r="L435" s="16" t="inlineStr">
         <is>
-          <t>Typed transition command and stable conflict errors implemented; recovery contracts remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Transition commands validate action/version and return stable 401/403/404/409 errors. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -27364,7 +27552,7 @@
       </c>
       <c r="J436" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K436" s="17" t="inlineStr">
@@ -27374,7 +27562,7 @@
       </c>
       <c r="L436" s="16" t="inlineStr">
         <is>
-          <t>Operator-only commands and owner-scoped buyer reads enforced; admin matrix remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Buyer owner projection, denied customer command and allowed operator are enforced. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -27426,7 +27614,7 @@
       </c>
       <c r="J437" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K437" s="17" t="inlineStr">
@@ -27436,7 +27624,7 @@
       </c>
       <c r="L437" s="16" t="inlineStr">
         <is>
-          <t>Conflict/invalid/missing paths fail closed; offline/retry expansion remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Loading/empty/unavailable/timeout/retry states are distinct and clear stale success. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -27488,7 +27676,7 @@
       </c>
       <c r="J438" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K438" s="17" t="inlineStr">
@@ -27498,7 +27686,7 @@
       </c>
       <c r="L438" s="16" t="inlineStr">
         <is>
-          <t>Append-only state and audit events include actor/action/target/time; reason/correlation remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Every transition has immutable state plus actor/reason/correlation/target audit metadata. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -27550,7 +27738,7 @@
       </c>
       <c r="J439" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K439" s="17" t="inlineStr">
@@ -27560,7 +27748,7 @@
       </c>
       <c r="L439" s="16" t="inlineStr">
         <is>
-          <t>Capability defaults off outside local test auth; dependency evidence remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Server flag defaults lifecycle simulation off outside isolated local mode. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -27612,7 +27800,7 @@
       </c>
       <c r="J440" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K440" s="17" t="inlineStr">
@@ -27622,7 +27810,7 @@
       </c>
       <c r="L440" s="16" t="inlineStr">
         <is>
-          <t>Deterministic full lifecycle fixture tested; failure/recovery fixtures remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Full success, stale version and invalid terminal fixtures are deterministic. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -27674,7 +27862,7 @@
       </c>
       <c r="J441" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K441" s="17" t="inlineStr">
@@ -27684,7 +27872,7 @@
       </c>
       <c r="L441" s="16" t="inlineStr">
         <is>
-          <t>Lifecycle and conflict rules covered in 17/17 suite; more boundary tests remain; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Lifecycle positive, boundary and denial rules execute in 18/18 suite. Shared evidence: docs/ai/SYNTHETIC-FLOW-CONTRACTS.md; strict typecheck; 18/18 unit/API tests; prior Chromium desktop/mobile flows; hosted capability fail-closed.</t>
         </is>
       </c>
     </row>
@@ -27736,7 +27924,7 @@
       </c>
       <c r="J442" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K442" s="17" t="inlineStr">
@@ -27746,7 +27934,7 @@
       </c>
       <c r="L442" s="16" t="inlineStr">
         <is>
-          <t>Local request/response/permission contracts pass; hosted disabled; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Local request/response/authorization/failure contracts execute; hosted local-only adapter is disabled and tested. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -27798,7 +27986,7 @@
       </c>
       <c r="J443" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K443" s="17" t="inlineStr">
@@ -27808,7 +27996,7 @@
       </c>
       <c r="L443" s="16" t="inlineStr">
         <is>
-          <t>Operator and buyer projections share append-only versions; hosted persistence pending; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Persistent records and connected projections agree on identifiers and versions. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -27860,7 +28048,7 @@
       </c>
       <c r="J444" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K444" s="17" t="inlineStr">
@@ -27870,7 +28058,7 @@
       </c>
       <c r="L444" s="16" t="inlineStr">
         <is>
-          <t>Chromium happy path passes; browser conflict/recovery capture remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Connected Chromium journey plus matching API denial assertions prove success and critical failure paths. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -27922,7 +28110,7 @@
       </c>
       <c r="J445" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K445" s="17" t="inlineStr">
@@ -27930,7 +28118,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L445" s="16" t="n"/>
+      <c r="L445" s="16" t="inlineStr">
+        <is>
+          <t>Semantic names, keyboard entry, reduced-motion and 320/tablet/desktop reflow pass; independent certification remains external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" s="16" t="inlineStr">
@@ -27980,7 +28172,7 @@
       </c>
       <c r="J446" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K446" s="17" t="inlineStr">
@@ -27988,7 +28180,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L446" s="16" t="n"/>
+      <c r="L446" s="16" t="inlineStr">
+        <is>
+          <t>Build artifacts meet 250 KiB entry and 30 KiB CSS engineering budgets; hosted Web Vitals remain external. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="16" t="inlineStr">
@@ -28038,7 +28234,7 @@
       </c>
       <c r="J447" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K447" s="17" t="inlineStr">
@@ -28048,7 +28244,7 @@
       </c>
       <c r="L447" s="16" t="inlineStr">
         <is>
-          <t>Role and stale-version escalation attempts fail; replay/injection expansion remains; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Cross-account/role/version escalation fails; secrets, tokens and document bytes are absent from client/audit data. Shared timeout/offline/unavailable/empty handling with explicit retry; typed contracts; 18/18 tests; prior connected Chromium evidence; docs/ai/SYNTHETIC-FLOW-CONTRACTS.md.</t>
         </is>
       </c>
     </row>
@@ -28100,7 +28296,7 @@
       </c>
       <c r="J448" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K448" s="17" t="inlineStr">
@@ -28108,7 +28304,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L448" s="16" t="n"/>
+      <c r="L448" s="16" t="inlineStr">
+        <is>
+          <t>Setup, flags, triage, recovery and bounded rollback are documented. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" s="16" t="inlineStr">
@@ -28158,7 +28358,7 @@
       </c>
       <c r="J449" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K449" s="17" t="inlineStr">
@@ -28166,7 +28366,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L449" s="16" t="n"/>
+      <c r="L449" s="16" t="inlineStr">
+        <is>
+          <t>Consent boundary and allowed/prohibited fields are documented; no telemetry transport is enabled. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" s="16" t="inlineStr">
@@ -28216,7 +28420,7 @@
       </c>
       <c r="J450" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K450" s="17" t="inlineStr">
@@ -28226,7 +28430,7 @@
       </c>
       <c r="L450" s="16" t="inlineStr">
         <is>
-          <t>Screenshots/tests captured; final commit and external boundary record pending; task/sr-passport-transitions; typecheck/build; test:unit 17/17; Chromium operator lifecycle + 390px checked-in Passport; synthetic only</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record in-progress closure evidence
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11899,7 +11899,7 @@
       </c>
       <c r="L175" s="16" t="inlineStr">
         <is>
-          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits. Content commit 6f7e370.</t>
         </is>
       </c>
     </row>
@@ -16330,7 +16330,7 @@
       </c>
       <c r="L250" s="16" t="inlineStr">
         <is>
-          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits. Content commit 6f7e370.</t>
         </is>
       </c>
     </row>
@@ -17871,7 +17871,7 @@
       </c>
       <c r="L275" s="16" t="inlineStr">
         <is>
-          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits. Content commit 6f7e370.</t>
         </is>
       </c>
     </row>
@@ -19412,7 +19412,7 @@
       </c>
       <c r="L300" s="16" t="inlineStr">
         <is>
-          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits. Content commit 6f7e370.</t>
         </is>
       </c>
     </row>
@@ -22398,7 +22398,7 @@
       </c>
       <c r="L350" s="16" t="inlineStr">
         <is>
-          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits. Content commit 6f7e370.</t>
         </is>
       </c>
     </row>
@@ -25444,7 +25444,7 @@
       </c>
       <c r="L400" s="16" t="inlineStr">
         <is>
-          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits. Content commit 6f7e370.</t>
         </is>
       </c>
     </row>
@@ -28430,7 +28430,7 @@
       </c>
       <c r="L450" s="16" t="inlineStr">
         <is>
-          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits.</t>
+          <t>Commands, results, browser evidence, performance budgets, rollback and external boundaries are recorded. docs/ai/SR-IN-PROGRESS-CLOSURE-QA.md; 18/18 tests; production builds; Chromium 320/768/1440 no-overflow, keyboard and reduced-motion checks; explicit hosted limits. Content commit 6f7e370.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record support recovery evidence
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28482,7 +28482,7 @@
       </c>
       <c r="J451" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K451" s="17" t="inlineStr">
@@ -28490,7 +28490,11 @@
           <t>All predecessors and required evidence pass, or the row remains blocked with a named reason and owner.</t>
         </is>
       </c>
-      <c r="L451" s="16" t="n"/>
+      <c r="L451" s="16" t="inlineStr">
+        <is>
+          <t>Accepted for isolated synthetic recovery only at content commit 7386cb6: owner-scoped support case and protected operator escalation/resolution extend the Passport recovery path; no real claim, refund, provider contact or production readiness. Typecheck/build pass; 19/19 tests; Chromium customer/operator flow.</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" s="16" t="inlineStr">
@@ -28535,7 +28539,7 @@
       </c>
       <c r="J452" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K452" s="17" t="inlineStr">
@@ -28543,7 +28547,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L452" s="16" t="n"/>
+      <c r="L452" s="16" t="inlineStr">
+        <is>
+          <t>Scope and gaps recorded in docs/exec-plans/SR-SUPPORT-RECOVERY.md at 7386cb6; routes/services/store are inventoried and notification delivery is explicitly absent.</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" s="16" t="inlineStr">
@@ -28593,7 +28601,7 @@
       </c>
       <c r="J453" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K453" s="17" t="inlineStr">
@@ -28601,7 +28609,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L453" s="16" t="n"/>
+      <c r="L453" s="16" t="inlineStr">
+        <is>
+          <t>Measurable local-only requirements, non-goals, hosted safety lock and communication gap recorded in docs/exec-plans/SR-SUPPORT-RECOVERY.md at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="16" t="inlineStr">
@@ -28651,7 +28663,7 @@
       </c>
       <c r="J454" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K454" s="17" t="inlineStr">
@@ -28659,7 +28671,11 @@
           <t>Fields, keys, owners, sensitivity, timestamps and lifecycle rules are explicit and use synthetic data only.</t>
         </is>
       </c>
-      <c r="L454" s="16" t="n"/>
+      <c r="L454" s="16" t="inlineStr">
+        <is>
+          <t>Typed SyntheticSupportCase plus SQLite owner/passport/category/status/version/UTC fields at 7386cb6; synthetic data only.</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" s="16" t="inlineStr">
@@ -28709,7 +28725,7 @@
       </c>
       <c r="J455" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K455" s="17" t="inlineStr">
@@ -28717,7 +28733,11 @@
           <t>Allowed and denied transitions are explicit; unknown, stale and conflicting inputs fail closed.</t>
         </is>
       </c>
-      <c r="L455" s="16" t="n"/>
+      <c r="L455" s="16" t="inlineStr">
+        <is>
+          <t>Open → escalated/resolved and escalated → resolved use expectedVersion; repeated, stale and terminal writes fail closed in 19/19 tests at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="16" t="inlineStr">
@@ -28767,7 +28787,7 @@
       </c>
       <c r="J456" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K456" s="17" t="inlineStr">
@@ -28775,7 +28795,11 @@
           <t>The principal route renders useful synthetic data, exposes no privileged data and does not imply a live transaction.</t>
         </is>
       </c>
-      <c r="L456" s="16" t="n"/>
+      <c r="L456" s="16" t="inlineStr">
+        <is>
+          <t>Customer /support and protected operations Support cases interfaces implemented at 7386cb6; constrained synthetic states and no live-message/refund claim.</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="16" t="inlineStr">
@@ -28825,7 +28849,7 @@
       </c>
       <c r="J457" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K457" s="17" t="inlineStr">
@@ -28833,7 +28857,11 @@
           <t>The route works at 320px, tablet and desktop widths without hidden actions, clipping or unusable controls.</t>
         </is>
       </c>
-      <c r="L457" s="16" t="n"/>
+      <c r="L457" s="16" t="inlineStr">
+        <is>
+          <t>Chromium verified /support at 320/768/1280 with scrollWidth equal viewport; touch controls remain &gt;=44px. Mobile persisted-case screenshot: /workspace/stayrelay-support-customer-mobile.png. Commit 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="16" t="inlineStr">
@@ -28883,7 +28911,7 @@
       </c>
       <c r="J458" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K458" s="17" t="inlineStr">
@@ -28891,7 +28919,11 @@
           <t>Components have typed inputs, accessible names and no direct authority over server-owned state.</t>
         </is>
       </c>
-      <c r="L458" s="16" t="n"/>
+      <c r="L458" s="16" t="inlineStr">
+        <is>
+          <t>Typed SupportCaseCard and typed category/options use shared domain contracts and design tokens; client invokes server commands only. Typecheck pass at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="16" t="inlineStr">
@@ -28941,7 +28973,7 @@
       </c>
       <c r="J459" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K459" s="17" t="inlineStr">
@@ -28949,7 +28981,11 @@
           <t>Invalid input is blocked with accessible guidance while server validation remains authoritative.</t>
         </is>
       </c>
-      <c r="L459" s="16" t="n"/>
+      <c r="L459" s="16" t="inlineStr">
+        <is>
+          <t>Constrained category select, owned optional Passport list, saving guard, inline failure/retry guidance; server revalidates every input. Commit 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" s="16" t="inlineStr">
@@ -28999,7 +29035,7 @@
       </c>
       <c r="J460" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K460" s="17" t="inlineStr">
@@ -29007,7 +29043,11 @@
           <t>Valid and invalid payloads return stable typed responses; missing authority returns a safe error.</t>
         </is>
       </c>
-      <c r="L460" s="16" t="n"/>
+      <c r="L460" s="16" t="inlineStr">
+        <is>
+          <t>Typed owner and operator request/response boundary with stable 400/401/403/404/409 failures; 19/19 API tests pass at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="16" t="inlineStr">
@@ -29057,7 +29097,7 @@
       </c>
       <c r="J461" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K461" s="17" t="inlineStr">
@@ -29065,7 +29105,11 @@
           <t>Owner, non-owner, allowed role, denied role and unauthenticated cases are tested server-side.</t>
         </is>
       </c>
-      <c r="L461" s="16" t="n"/>
+      <c r="L461" s="16" t="inlineStr">
+        <is>
+          <t>Anonymous, non-owner Passport, customer-to-operator, owner read and operator transition cases execute server-side in 19/19 tests at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="16" t="inlineStr">
@@ -29115,7 +29159,7 @@
       </c>
       <c r="J462" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K462" s="17" t="inlineStr">
@@ -29123,7 +29167,11 @@
           <t>Loading, empty, unavailable, timeout and retry states are distinguishable and never expose stale success.</t>
         </is>
       </c>
-      <c r="L462" s="16" t="n"/>
+      <c r="L462" s="16" t="inlineStr">
+        <is>
+          <t>Distinct loading, empty, hosted-disabled/timeout-safe, failed-save and retry states never project stale success. Chromium unavailable reflow plus connected flow at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="463">
       <c r="A463" s="16" t="inlineStr">
@@ -29173,7 +29221,7 @@
       </c>
       <c r="J463" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K463" s="17" t="inlineStr">
@@ -29181,7 +29229,11 @@
           <t>Privileged actions produce immutable-shaped events with actor, reason, correlation and target metadata.</t>
         </is>
       </c>
-      <c r="L463" s="16" t="n"/>
+      <c r="L463" s="16" t="inlineStr">
+        <is>
+          <t>Create/escalate/resolve commands append actor/action/reason/correlation/target/UTC audit metadata without free text or document content. Tests pass at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" s="16" t="inlineStr">
@@ -29231,7 +29283,7 @@
       </c>
       <c r="J464" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K464" s="17" t="inlineStr">
@@ -29239,7 +29291,11 @@
           <t>The capability is off by default where required and cannot be enabled from client code.</t>
         </is>
       </c>
-      <c r="L464" s="16" t="n"/>
+      <c r="L464" s="16" t="inlineStr">
+        <is>
+          <t>STAYRELAY_TEST_AUTH remains server-owned and default-off; hosted UI explains disabled state and cannot enable it. Disabled-adapter test passes at 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="465">
       <c r="A465" s="16" t="inlineStr">
@@ -29405,7 +29461,7 @@
       </c>
       <c r="J467" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K467" s="17" t="inlineStr">
@@ -29413,7 +29469,11 @@
           <t>Request, response, authorization and failure contracts execute against both local and hosted adapters where applicable.</t>
         </is>
       </c>
-      <c r="L467" s="16" t="n"/>
+      <c r="L467" s="16" t="inlineStr">
+        <is>
+          <t>Contract suite at 7386cb6 covers invalid category, anonymous denial, cross-account Passport denial, operator-role denial, stale version and terminal replay; local adapter passes and hosted adapter stays disabled.</t>
+        </is>
+      </c>
     </row>
     <row r="468">
       <c r="A468" s="16" t="inlineStr">
@@ -29579,7 +29639,7 @@
       </c>
       <c r="J470" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K470" s="17" t="inlineStr">
@@ -29587,7 +29647,11 @@
           <t>Keyboard, focus, semantic naming, contrast, reflow and reduced-motion checks have recorded results.</t>
         </is>
       </c>
-      <c r="L470" s="16" t="n"/>
+      <c r="L470" s="16" t="inlineStr">
+        <is>
+          <t>Chromium keyboard focus and semantic-label checks plus 320/768/1280 no-overflow reflow pass; shared token contrast/reduced-motion rules retained. Independent certification remains external. Commit 7386cb6.</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Record support feed validation and next checkpoint
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,8 +1544,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -29345,7 +29345,7 @@
       </c>
       <c r="J465" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K465" s="17" t="inlineStr">
@@ -29353,7 +29353,11 @@
           <t>Fixtures are deterministic, visibly fictional and include positive and negative states without real personal data.</t>
         </is>
       </c>
-      <c r="L465" s="16" t="n"/>
+      <c r="L465" s="16" t="inlineStr">
+        <is>
+          <t>Deterministic synthetic support success/denial/stale/terminal/audit-failure scenarios and bounded owner feed fixtures. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" s="16" t="inlineStr">
@@ -29403,7 +29407,7 @@
       </c>
       <c r="J466" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K466" s="17" t="inlineStr">
@@ -29411,7 +29415,11 @@
           <t>Focused tests execute and cover core positive, boundary and denial rules.</t>
         </is>
       </c>
-      <c r="L466" s="16" t="n"/>
+      <c r="L466" s="16" t="inlineStr">
+        <is>
+          <t>22 tests pass, including injected audit rollback and stale retry rules. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" s="16" t="inlineStr">
@@ -29523,7 +29531,7 @@
       </c>
       <c r="J468" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K468" s="17" t="inlineStr">
@@ -29531,7 +29539,11 @@
           <t>Persisted synthetic state survives reload and connected projections agree on identifiers and versions.</t>
         </is>
       </c>
-      <c r="L468" s="16" t="n"/>
+      <c r="L468" s="16" t="inlineStr">
+        <is>
+          <t>On-disk SQLite reopened across independent connections; case state and owner feed persist and remain isolated. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="469">
       <c r="A469" s="16" t="inlineStr">
@@ -29581,7 +29593,7 @@
       </c>
       <c r="J469" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K469" s="17" t="inlineStr">
@@ -29589,7 +29601,11 @@
           <t>Browser evidence and matching API/data assertions prove the main path and at least one failure path.</t>
         </is>
       </c>
-      <c r="L469" s="16" t="n"/>
+      <c r="L469" s="16" t="inlineStr">
+        <is>
+          <t>Chromium customer create → operator escalate/resolve → customer refresh; offline refresh clears stale feed and exposes retry. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" s="16" t="inlineStr">
@@ -29701,7 +29717,7 @@
       </c>
       <c r="J471" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K471" s="17" t="inlineStr">
@@ -29709,7 +29725,11 @@
           <t>Recorded measurements meet a stated budget or retain an explicit remediation blocker.</t>
         </is>
       </c>
-      <c r="L471" s="16" t="n"/>
+      <c r="L471" s="16" t="inlineStr">
+        <is>
+          <t>Measured build entry 214.70 kB &lt; 250 KiB and CSS 21.79 kB &lt; 30 KiB; support route 5.18 kB. Hosted Web Vitals remain unverified. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" s="16" t="inlineStr">
@@ -29759,7 +29779,7 @@
       </c>
       <c r="J472" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K472" s="17" t="inlineStr">
@@ -29767,7 +29787,11 @@
           <t>Cross-account and role escalation attempts fail; secrets and sensitive contents are absent from client and logs.</t>
         </is>
       </c>
-      <c r="L472" s="16" t="n"/>
+      <c r="L472" s="16" t="inlineStr">
+        <is>
+          <t>Owner-feed exclusion, exact field allowlist, stale/repeated transition denial and audit-failure rollback verified. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" s="16" t="inlineStr">
@@ -29817,7 +29841,7 @@
       </c>
       <c r="J473" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K473" s="17" t="inlineStr">
@@ -29825,7 +29849,11 @@
           <t>A new contributor can start, verify, diagnose, recover and roll back the capability from the guide.</t>
         </is>
       </c>
-      <c r="L473" s="16" t="n"/>
+      <c r="L473" s="16" t="inlineStr">
+        <is>
+          <t>Runnable local startup, operator workflow, failure triage, retry and rollback documented. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="474">
       <c r="A474" s="16" t="inlineStr">
@@ -29875,7 +29903,7 @@
       </c>
       <c r="J474" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K474" s="17" t="inlineStr">
@@ -29883,7 +29911,11 @@
           <t>Allowed events, consent/context and forbidden sensitive fields are documented and tested.</t>
         </is>
       </c>
-      <c r="L474" s="16" t="n"/>
+      <c r="L474" s="16" t="inlineStr">
+        <is>
+          <t>Operational event allowlist and excluded sensitive fields documented and asserted; no analytics or external messaging transport. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" s="16" t="inlineStr">
@@ -29933,7 +29965,7 @@
       </c>
       <c r="J475" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K475" s="17" t="inlineStr">
@@ -29941,7 +29973,11 @@
           <t>Evidence names exact commit, environment, commands, results and unverified external boundaries.</t>
         </is>
       </c>
-      <c r="L475" s="16" t="n"/>
+      <c r="L475" s="16" t="inlineStr">
+        <is>
+          <t>Content commit, local commands/results, Chromium screenshot, bundle budgets and boundaries recorded. Content 859197c; docs/ai/SR-SUPPORT-FEED-QA.md; tests/unit/supportPersistence.test.ts. Completion covers support and in-app case updates; external delivery/preferences remain acceptance gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" s="16" t="inlineStr">
@@ -29991,7 +30027,7 @@
       </c>
       <c r="J476" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K476" s="17" t="inlineStr">
@@ -29999,7 +30035,11 @@
           <t>All predecessors and required evidence pass, or the row remains blocked with a named reason and owner.</t>
         </is>
       </c>
-      <c r="L476" s="16" t="n"/>
+      <c r="L476" s="16" t="inlineStr">
+        <is>
+          <t>Support and in-app feed checks pass at 859197c. Acceptance remains open: notification preferences, disconnected delivery adapter/retries, and required review are unfinished. Next implement notification delivery simulation.</t>
+        </is>
+      </c>
     </row>
     <row r="477">
       <c r="A477" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Close synthetic support notification acceptance
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30027,7 +30027,7 @@
       </c>
       <c r="J476" s="17" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K476" s="17" t="inlineStr">
@@ -30037,7 +30037,7 @@
       </c>
       <c r="L476" s="16" t="inlineStr">
         <is>
-          <t>Support and in-app feed checks pass at 859197c. Acceptance remains open: notification preferences, disconnected delivery adapter/retries, and required review are unfinished. Next implement notification delivery simulation.</t>
+          <t>Synthetic Part 19 acceptance passes at content commit 45aad56: support cases, owner activity feed, versioned in-app preference, disconnected delivery outcomes and failure/retry tests are evidenced. External email/SMS/push/webhook delivery, hosted persistence and independent certification remain blocked and disabled. See docs/ai/SR-SUPPORT-FEED-QA.md; 23/23 tests; strict typecheck/build; Chromium 390px preference flow.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record recovery flow acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28492,7 +28492,7 @@
       </c>
       <c r="L451" s="16" t="inlineStr">
         <is>
-          <t>Accepted for isolated synthetic recovery only at content commit 7386cb6: owner-scoped support case and protected operator escalation/resolution extend the Passport recovery path; no real claim, refund, provider contact or production readiness. Typecheck/build pass; 19/19 tests; Chromium customer/operator flow.</t>
+          <t>Acceptance evidence expanded at content commit d00a5a2: support and synthetic cancellation/refund/recovery flows pass owner, seller, operator, audit, version and no-payment checks. 24/24 tests; strict typecheck/build; Chromium buyer 390px and operations recovery queue 1280px. docs/ai/SR-RECOVERY-FLOW-QA.md. External refunds, payout, provider delivery and hosted persistence remain disabled.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record durability evidence and working Vercel proxy access
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,8 +1544,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -28492,7 +28492,7 @@
       </c>
       <c r="L451" s="16" t="inlineStr">
         <is>
-          <t>Acceptance evidence expanded at content commit d00a5a2: support and synthetic cancellation/refund/recovery flows pass owner, seller, operator, audit, version and no-payment checks. 24/24 tests; strict typecheck/build; Chromium buyer 390px and operations recovery queue 1280px. docs/ai/SR-RECOVERY-FLOW-QA.md. External refunds, payout, provider delivery and hosted persistence remain disabled.</t>
+          <t>Acceptance evidence expanded at content commit d00a5a2: support and synthetic cancellation/refund/recovery flows pass owner, seller, operator, audit, version and no-payment checks. 24/24 tests; strict typecheck/build; Chromium buyer 390px and operations recovery queue 1280px. docs/ai/SR-RECOVERY-FLOW-QA.md. External refunds, payout, provider delivery and hosted persistence remain disabled. | Durability repair 12dc050 / 1f1f511: 27 tests and builds pass; docs/ai/SR-RECOVERY-DURABILITY-QA.md. Broad package acceptance remains partial: recovery draft/timeline and notification feed enforcement not verified. No new completion claimed.</t>
         </is>
       </c>
     </row>
@@ -30037,7 +30037,7 @@
       </c>
       <c r="L476" s="16" t="inlineStr">
         <is>
-          <t>Synthetic Part 19 acceptance passes at content commit 45aad56: support cases, owner activity feed, versioned in-app preference, disconnected delivery outcomes and failure/retry tests are evidenced. External email/SMS/push/webhook delivery, hosted persistence and independent certification remain blocked and disabled. See docs/ai/SR-SUPPORT-FEED-QA.md; 23/23 tests; strict typecheck/build; Chromium 390px preference flow.</t>
+          <t>Synthetic Part 19 acceptance passes at content commit 45aad56: support cases, owner activity feed, versioned in-app preference, disconnected delivery outcomes and failure/retry tests are evidenced. External email/SMS/push/webhook delivery, hosted persistence and independent certification remain blocked and disabled. See docs/ai/SR-SUPPORT-FEED-QA.md; 23/23 tests; strict typecheck/build; Chromium 390px preference flow. | Durability repair 12dc050 / 1f1f511: 27 tests and builds pass; docs/ai/SR-RECOVERY-DURABILITY-QA.md. Broad package acceptance remains partial: recovery draft/timeline and notification feed enforcement not verified. No new completion claimed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Save selection and preference verification checkpoint
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28492,7 +28492,7 @@
       </c>
       <c r="L451" s="16" t="inlineStr">
         <is>
-          <t>Acceptance evidence expanded at content commit d00a5a2: support and synthetic cancellation/refund/recovery flows pass owner, seller, operator, audit, version and no-payment checks. 24/24 tests; strict typecheck/build; Chromium buyer 390px and operations recovery queue 1280px. docs/ai/SR-RECOVERY-FLOW-QA.md. External refunds, payout, provider delivery and hosted persistence remain disabled. | Durability repair 12dc050 / 1f1f511: 27 tests and builds pass; docs/ai/SR-RECOVERY-DURABILITY-QA.md. Broad package acceptance remains partial: recovery draft/timeline and notification feed enforcement not verified. No new completion claimed.</t>
+          <t>Acceptance evidence expanded at content commit d00a5a2: support and synthetic cancellation/refund/recovery flows pass owner, seller, operator, audit, version and no-payment checks. 24/24 tests; strict typecheck/build; Chromium buyer 390px and operations recovery queue 1280px. docs/ai/SR-RECOVERY-FLOW-QA.md. External refunds, payout, provider delivery and hosted persistence remain disabled. | Durability repair 12dc050 / 1f1f511: 27 tests and builds pass; docs/ai/SR-RECOVERY-DURABILITY-QA.md. Broad package acceptance remains partial: recovery draft/timeline and notification feed enforcement not verified. No new completion claimed. | a7b88dd: explicit recovery Passport selection and server-enforced feed preference; 27 tests/builds and browser contract checks. docs/ai/SR-SELECTION-PREFERENCE-QA.md. Broader package gaps remain.</t>
         </is>
       </c>
     </row>
@@ -30037,7 +30037,7 @@
       </c>
       <c r="L476" s="16" t="inlineStr">
         <is>
-          <t>Synthetic Part 19 acceptance passes at content commit 45aad56: support cases, owner activity feed, versioned in-app preference, disconnected delivery outcomes and failure/retry tests are evidenced. External email/SMS/push/webhook delivery, hosted persistence and independent certification remain blocked and disabled. See docs/ai/SR-SUPPORT-FEED-QA.md; 23/23 tests; strict typecheck/build; Chromium 390px preference flow. | Durability repair 12dc050 / 1f1f511: 27 tests and builds pass; docs/ai/SR-RECOVERY-DURABILITY-QA.md. Broad package acceptance remains partial: recovery draft/timeline and notification feed enforcement not verified. No new completion claimed.</t>
+          <t>Synthetic Part 19 acceptance passes at content commit 45aad56: support cases, owner activity feed, versioned in-app preference, disconnected delivery outcomes and failure/retry tests are evidenced. External email/SMS/push/webhook delivery, hosted persistence and independent certification remain blocked and disabled. See docs/ai/SR-SUPPORT-FEED-QA.md; 23/23 tests; strict typecheck/build; Chromium 390px preference flow. | Durability repair 12dc050 / 1f1f511: 27 tests and builds pass; docs/ai/SR-RECOVERY-DURABILITY-QA.md. Broad package acceptance remains partial: recovery draft/timeline and notification feed enforcement not verified. No new completion claimed. | a7b88dd: explicit recovery Passport selection and server-enforced feed preference; 27 tests/builds and browser contract checks. docs/ai/SR-SELECTION-PREFERENCE-QA.md. Broader package gaps remain.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record test contracts, remote validation and continuation checkpoint
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,9 +1544,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -35864,7 +35864,7 @@
       </c>
       <c r="J577" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K577" s="17" t="inlineStr">
@@ -35872,7 +35872,11 @@
           <t>Existing implementation, reusable evidence, gaps and prohibited assumptions are enumerated with repository paths.</t>
         </is>
       </c>
-      <c r="L577" s="16" t="n"/>
+      <c r="L577" s="16" t="inlineStr">
+        <is>
+          <t>a219d54; docs/ai/SR-TEST-COVERAGE-CONTRACT.md: repository coverage audit and measurable test contract. 27 local tests and both builds/typecheck pass. Remote CI result tracked separately; no broad test-package completion.</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" s="16" t="inlineStr">
@@ -35922,7 +35926,7 @@
       </c>
       <c r="J578" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K578" s="17" t="inlineStr">
@@ -35930,7 +35934,11 @@
           <t>Requirements are measurable, preserve server authority and distinguish implemented, simulated, disconnected and blocked behavior.</t>
         </is>
       </c>
-      <c r="L578" s="16" t="n"/>
+      <c r="L578" s="16" t="inlineStr">
+        <is>
+          <t>a219d54; docs/ai/SR-TEST-COVERAGE-CONTRACT.md: repository coverage audit and measurable test contract. 27 local tests and both builds/typecheck pass. Remote CI result tracked separately; no broad test-package completion.</t>
+        </is>
+      </c>
     </row>
     <row r="579">
       <c r="A579" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Save verified public demo release and remaining backend boundaries
</commit_message>
<xml_diff>
--- a/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
+++ b/docs/project-control/StayRelay_750_Task_Supplemental_Tracker.xlsx
@@ -1544,8 +1544,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -45942,7 +45942,11 @@
           <t>All predecessors and required evidence pass, or the row remains blocked with a named reason and owner.</t>
         </is>
       </c>
-      <c r="L751" s="16" t="n"/>
+      <c r="L751" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Partial release evidence only: public synthetic frontend deployed ce906b0; docs/ai/SR-PUBLIC-DEMO-RELEASE.md; hosted browser and fail-closed JSON smoke pass. Hosted backend and remaining scope incomplete; acceptance NOT closed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L751"/>

</xml_diff>